<commit_message>
ajouts logos et tests
</commit_message>
<xml_diff>
--- a/Data/FairCarboN_Datas_Labo2.xlsx
+++ b/Data/FairCarboN_Datas_Labo2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8EC5B98-89C9-450E-8FBC-A3EFAB7FF091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{011C1A7A-9A31-4606-A589-A1247AE57B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4435,9 +4435,6 @@
     <t>Pays</t>
   </si>
   <si>
-    <t>logos</t>
-  </si>
-  <si>
     <t>France</t>
   </si>
   <si>
@@ -4466,6 +4463,9 @@
   </si>
   <si>
     <t>Zimbabwe</t>
+  </si>
+  <si>
+    <t>Logos</t>
   </si>
 </sst>
 </file>
@@ -5048,7 +5048,7 @@
         <v>1434</v>
       </c>
       <c r="O1" s="31" t="s">
-        <v>1435</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="93.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -5092,7 +5092,7 @@
         <v>78</v>
       </c>
       <c r="N2" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O2" s="23" t="str">
         <f>"DATA/logos/" &amp; TEXT(E2,"jjj") &amp; ".png"</f>
@@ -5140,7 +5140,7 @@
         <v>170</v>
       </c>
       <c r="N3" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O3" s="23" t="str">
         <f t="shared" ref="O3:O66" si="0">"DATA/logos/" &amp; TEXT(E3,"jjj") &amp; ".png"</f>
@@ -5188,7 +5188,7 @@
         <v>170</v>
       </c>
       <c r="N4" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O4" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5234,7 +5234,7 @@
         <v>162</v>
       </c>
       <c r="N5" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O5" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5280,7 +5280,7 @@
         <v>162</v>
       </c>
       <c r="N6" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O6" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5374,7 +5374,7 @@
         <v>111</v>
       </c>
       <c r="N8" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O8" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5422,7 +5422,7 @@
         <v>12</v>
       </c>
       <c r="N9" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O9" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5470,7 +5470,7 @@
         <v>12</v>
       </c>
       <c r="N10" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O10" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5518,7 +5518,7 @@
         <v>212</v>
       </c>
       <c r="N11" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O11" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5566,14 +5566,14 @@
         <v>212</v>
       </c>
       <c r="N12" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O12" s="23" t="str">
         <f t="shared" si="0"/>
         <v>DATA/logos/AMAP.png</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" ht="31" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
@@ -5700,7 +5700,7 @@
         <v>19</v>
       </c>
       <c r="N15" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O15" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5746,7 +5746,7 @@
         <v>19</v>
       </c>
       <c r="N16" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O16" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5792,7 +5792,7 @@
         <v>19</v>
       </c>
       <c r="N17" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O17" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5838,7 +5838,7 @@
         <v>19</v>
       </c>
       <c r="N18" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O18" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5884,7 +5884,7 @@
         <v>19</v>
       </c>
       <c r="N19" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O19" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5928,7 +5928,7 @@
         <v>449</v>
       </c>
       <c r="N20" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O20" s="23" t="str">
         <f t="shared" si="0"/>
@@ -5976,7 +5976,7 @@
         <v>417</v>
       </c>
       <c r="N21" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O21" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6024,7 +6024,7 @@
         <v>417</v>
       </c>
       <c r="N22" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O22" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6072,7 +6072,7 @@
         <v>417</v>
       </c>
       <c r="N23" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O23" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6120,7 +6120,7 @@
         <v>32</v>
       </c>
       <c r="N24" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O24" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6168,7 +6168,7 @@
         <v>32</v>
       </c>
       <c r="N25" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O25" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6216,7 +6216,7 @@
         <v>5.4070900000000002</v>
       </c>
       <c r="N26" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O26" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6258,7 +6258,7 @@
         <v>555</v>
       </c>
       <c r="N27" s="32" t="s">
-        <v>1437</v>
+        <v>1436</v>
       </c>
       <c r="O27" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6304,7 +6304,7 @@
         <v>233</v>
       </c>
       <c r="N28" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O28" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6350,14 +6350,14 @@
         <v>233</v>
       </c>
       <c r="N29" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O29" s="23" t="str">
         <f t="shared" si="0"/>
         <v>DATA/logos/BOREA.png</v>
       </c>
     </row>
-    <row r="30" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" ht="31" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>7</v>
       </c>
@@ -6392,7 +6392,7 @@
         <v>565</v>
       </c>
       <c r="N30" s="32" t="s">
-        <v>1438</v>
+        <v>1437</v>
       </c>
       <c r="O30" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6432,7 +6432,7 @@
         <v>456</v>
       </c>
       <c r="N31" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O31" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6478,7 +6478,7 @@
         <v>129</v>
       </c>
       <c r="N32" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O32" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6524,7 +6524,7 @@
         <v>129</v>
       </c>
       <c r="N33" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O33" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6572,7 +6572,7 @@
         <v>303</v>
       </c>
       <c r="N34" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O34" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6620,7 +6620,7 @@
         <v>181</v>
       </c>
       <c r="N35" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O35" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6666,7 +6666,7 @@
         <v>134</v>
       </c>
       <c r="N36" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O36" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6712,7 +6712,7 @@
         <v>425</v>
       </c>
       <c r="N37" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O37" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6758,7 +6758,7 @@
         <v>26</v>
       </c>
       <c r="N38" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O38" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6804,7 +6804,7 @@
         <v>26</v>
       </c>
       <c r="N39" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O39" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6850,7 +6850,7 @@
         <v>398</v>
       </c>
       <c r="N40" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O40" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6896,7 +6896,7 @@
         <v>191</v>
       </c>
       <c r="N41" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O41" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6942,7 +6942,7 @@
         <v>191</v>
       </c>
       <c r="N42" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O42" s="23" t="str">
         <f t="shared" si="0"/>
@@ -6988,7 +6988,7 @@
         <v>378</v>
       </c>
       <c r="N43" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O43" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7034,7 +7034,7 @@
         <v>378</v>
       </c>
       <c r="N44" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O44" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7082,7 +7082,7 @@
         <v>314</v>
       </c>
       <c r="N45" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O45" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7130,7 +7130,7 @@
         <v>429</v>
       </c>
       <c r="N46" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O46" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7178,7 +7178,7 @@
         <v>303</v>
       </c>
       <c r="N47" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O47" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7226,7 +7226,7 @@
         <v>303</v>
       </c>
       <c r="N48" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O48" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7274,7 +7274,7 @@
         <v>303</v>
       </c>
       <c r="N49" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O49" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7322,7 +7322,7 @@
         <v>303</v>
       </c>
       <c r="N50" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O50" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7370,7 +7370,7 @@
         <v>303</v>
       </c>
       <c r="N51" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O51" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7418,7 +7418,7 @@
         <v>303</v>
       </c>
       <c r="N52" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O52" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7466,7 +7466,7 @@
         <v>303</v>
       </c>
       <c r="N53" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O53" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7514,7 +7514,7 @@
         <v>616</v>
       </c>
       <c r="N54" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O54" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7560,7 +7560,7 @@
         <v>434</v>
       </c>
       <c r="N55" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O55" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7608,7 +7608,7 @@
         <v>32</v>
       </c>
       <c r="N56" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O56" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7656,7 +7656,7 @@
         <v>32</v>
       </c>
       <c r="N57" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O57" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7704,7 +7704,7 @@
         <v>32</v>
       </c>
       <c r="N58" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O58" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7752,7 +7752,7 @@
         <v>32</v>
       </c>
       <c r="N59" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O59" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7800,14 +7800,14 @@
         <v>32</v>
       </c>
       <c r="N60" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O60" s="23" t="str">
         <f t="shared" si="0"/>
         <v>DATA/logos/ECOSYS.png</v>
       </c>
     </row>
-    <row r="61" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>7</v>
       </c>
@@ -7842,7 +7842,7 @@
         <v>628</v>
       </c>
       <c r="N61" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O61" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7890,7 +7890,7 @@
         <v>144</v>
       </c>
       <c r="N62" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O62" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7938,7 +7938,7 @@
         <v>144</v>
       </c>
       <c r="N63" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O63" s="23" t="str">
         <f t="shared" si="0"/>
@@ -7986,7 +7986,7 @@
         <v>237</v>
       </c>
       <c r="N64" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O64" s="23" t="str">
         <f t="shared" si="0"/>
@@ -8034,7 +8034,7 @@
         <v>237</v>
       </c>
       <c r="N65" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O65" s="23" t="str">
         <f t="shared" si="0"/>
@@ -8080,7 +8080,7 @@
         <v>646</v>
       </c>
       <c r="N66" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O66" s="23" t="str">
         <f t="shared" si="0"/>
@@ -8126,7 +8126,7 @@
         <v>646</v>
       </c>
       <c r="N67" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O67" s="23" t="str">
         <f t="shared" ref="O67:O130" si="1">"DATA/logos/" &amp; TEXT(E67,"jjj") &amp; ".png"</f>
@@ -8172,7 +8172,7 @@
         <v>646</v>
       </c>
       <c r="N68" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O68" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8220,7 +8220,7 @@
         <v>414</v>
       </c>
       <c r="N69" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O69" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8268,7 +8268,7 @@
         <v>414</v>
       </c>
       <c r="N70" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O70" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8316,7 +8316,7 @@
         <v>239</v>
       </c>
       <c r="N71" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O71" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8364,7 +8364,7 @@
         <v>239</v>
       </c>
       <c r="N72" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O72" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8412,7 +8412,7 @@
         <v>239</v>
       </c>
       <c r="N73" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O73" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8460,7 +8460,7 @@
         <v>402</v>
       </c>
       <c r="N74" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O74" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8506,7 +8506,7 @@
         <v>364</v>
       </c>
       <c r="N75" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O75" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8552,7 +8552,7 @@
         <v>193</v>
       </c>
       <c r="N76" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O76" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8596,7 +8596,7 @@
         <v>353</v>
       </c>
       <c r="N77" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O77" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8644,7 +8644,7 @@
         <v>350</v>
       </c>
       <c r="N78" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O78" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8692,7 +8692,7 @@
         <v>350</v>
       </c>
       <c r="N79" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O79" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8738,7 +8738,7 @@
         <v>202</v>
       </c>
       <c r="N80" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O80" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8784,7 +8784,7 @@
         <v>202</v>
       </c>
       <c r="N81" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O81" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8830,7 +8830,7 @@
         <v>202</v>
       </c>
       <c r="N82" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O82" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8878,7 +8878,7 @@
         <v>218</v>
       </c>
       <c r="N83" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O83" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8926,7 +8926,7 @@
         <v>346</v>
       </c>
       <c r="N84" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O84" s="23" t="str">
         <f t="shared" si="1"/>
@@ -8974,7 +8974,7 @@
         <v>243</v>
       </c>
       <c r="N85" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O85" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9022,7 +9022,7 @@
         <v>372</v>
       </c>
       <c r="N86" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O86" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9070,7 +9070,7 @@
         <v>372</v>
       </c>
       <c r="N87" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O87" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9118,7 +9118,7 @@
         <v>372</v>
       </c>
       <c r="N88" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O88" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9166,7 +9166,7 @@
         <v>372</v>
       </c>
       <c r="N89" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O89" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9214,7 +9214,7 @@
         <v>372</v>
       </c>
       <c r="N90" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O90" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9308,7 +9308,7 @@
         <v>372</v>
       </c>
       <c r="N92" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O92" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9356,7 +9356,7 @@
         <v>222</v>
       </c>
       <c r="N93" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O93" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9404,7 +9404,7 @@
         <v>222</v>
       </c>
       <c r="N94" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O94" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9452,7 +9452,7 @@
         <v>222</v>
       </c>
       <c r="N95" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O95" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9500,7 +9500,7 @@
         <v>222</v>
       </c>
       <c r="N96" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O96" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9548,7 +9548,7 @@
         <v>419</v>
       </c>
       <c r="N97" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O97" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9596,7 +9596,7 @@
         <v>383</v>
       </c>
       <c r="N98" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O98" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9642,7 +9642,7 @@
         <v>445</v>
       </c>
       <c r="N99" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O99" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9688,14 +9688,14 @@
         <v>337</v>
       </c>
       <c r="N100" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O100" s="23" t="str">
         <f t="shared" si="1"/>
         <v>DATA/logos/Info&amp;Sols.png</v>
       </c>
     </row>
-    <row r="101" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>7</v>
       </c>
@@ -9730,7 +9730,7 @@
         <v>709</v>
       </c>
       <c r="N101" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O101" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9778,7 +9778,7 @@
         <v>353</v>
       </c>
       <c r="N102" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O102" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9826,7 +9826,7 @@
         <v>353</v>
       </c>
       <c r="N103" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O103" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9874,7 +9874,7 @@
         <v>249</v>
       </c>
       <c r="N104" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O104" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9922,7 +9922,7 @@
         <v>392</v>
       </c>
       <c r="N105" s="1" t="s">
-        <v>1439</v>
+        <v>1438</v>
       </c>
       <c r="O105" s="23" t="str">
         <f t="shared" si="1"/>
@@ -9970,7 +9970,7 @@
         <v>374</v>
       </c>
       <c r="N106" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O106" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10018,7 +10018,7 @@
         <v>106</v>
       </c>
       <c r="N107" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O107" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10066,7 +10066,7 @@
         <v>106</v>
       </c>
       <c r="N108" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O108" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10160,7 +10160,7 @@
         <v>339</v>
       </c>
       <c r="N110" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O110" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10208,7 +10208,7 @@
         <v>339</v>
       </c>
       <c r="N111" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O111" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10256,7 +10256,7 @@
         <v>372</v>
       </c>
       <c r="N112" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O112" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10304,7 +10304,7 @@
         <v>372</v>
       </c>
       <c r="N113" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O113" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10352,7 +10352,7 @@
         <v>372</v>
       </c>
       <c r="N114" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O114" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10400,7 +10400,7 @@
         <v>356</v>
       </c>
       <c r="N115" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O115" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10448,7 +10448,7 @@
         <v>358</v>
       </c>
       <c r="N116" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O116" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10496,7 +10496,7 @@
         <v>358</v>
       </c>
       <c r="N117" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O117" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10542,7 +10542,7 @@
         <v>254</v>
       </c>
       <c r="N118" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O118" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10590,7 +10590,7 @@
         <v>491</v>
       </c>
       <c r="N119" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O119" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10638,7 +10638,7 @@
         <v>491</v>
       </c>
       <c r="N120" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O120" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10684,7 +10684,7 @@
         <v>258</v>
       </c>
       <c r="N121" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O121" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10732,7 +10732,7 @@
         <v>438</v>
       </c>
       <c r="N122" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O122" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10780,7 +10780,7 @@
         <v>137</v>
       </c>
       <c r="N123" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O123" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10828,7 +10828,7 @@
         <v>137</v>
       </c>
       <c r="N124" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O124" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10876,7 +10876,7 @@
         <v>348</v>
       </c>
       <c r="N125" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O125" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10924,7 +10924,7 @@
         <v>348</v>
       </c>
       <c r="N126" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O126" s="23" t="str">
         <f t="shared" si="1"/>
@@ -10972,7 +10972,7 @@
         <v>308</v>
       </c>
       <c r="N127" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O127" s="23" t="str">
         <f t="shared" si="1"/>
@@ -11020,7 +11020,7 @@
         <v>86</v>
       </c>
       <c r="N128" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O128" s="23" t="str">
         <f t="shared" si="1"/>
@@ -11068,7 +11068,7 @@
         <v>86</v>
       </c>
       <c r="N129" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O129" s="23" t="str">
         <f t="shared" si="1"/>
@@ -11112,7 +11112,7 @@
         <v>773</v>
       </c>
       <c r="N130" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O130" s="23" t="str">
         <f t="shared" si="1"/>
@@ -11160,7 +11160,7 @@
         <v>263</v>
       </c>
       <c r="N131" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O131" s="23" t="str">
         <f t="shared" ref="O131:O194" si="2">"DATA/logos/" &amp; TEXT(E131,"jjj") &amp; ".png"</f>
@@ -11208,7 +11208,7 @@
         <v>265</v>
       </c>
       <c r="N132" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O132" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11254,7 +11254,7 @@
         <v>267</v>
       </c>
       <c r="N133" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O133" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11300,7 +11300,7 @@
         <v>267</v>
       </c>
       <c r="N134" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O134" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11346,7 +11346,7 @@
         <v>267</v>
       </c>
       <c r="N135" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O135" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11392,7 +11392,7 @@
         <v>267</v>
       </c>
       <c r="N136" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O136" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11438,7 +11438,7 @@
         <v>267</v>
       </c>
       <c r="N137" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O137" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11484,7 +11484,7 @@
         <v>267</v>
       </c>
       <c r="N138" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O138" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11530,7 +11530,7 @@
         <v>267</v>
       </c>
       <c r="N139" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O139" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11578,7 +11578,7 @@
         <v>271</v>
       </c>
       <c r="N140" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O140" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11624,7 +11624,7 @@
         <v>456</v>
       </c>
       <c r="N141" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O141" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11670,7 +11670,7 @@
         <v>456</v>
       </c>
       <c r="N142" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O142" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11712,7 +11712,7 @@
         <v>342</v>
       </c>
       <c r="N143" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O143" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11760,7 +11760,7 @@
         <v>800</v>
       </c>
       <c r="N144" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O144" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11806,7 +11806,7 @@
         <v>370</v>
       </c>
       <c r="N145" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O145" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11852,7 +11852,7 @@
         <v>370</v>
       </c>
       <c r="N146" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O146" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11898,7 +11898,7 @@
         <v>370</v>
       </c>
       <c r="N147" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O147" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11944,7 +11944,7 @@
         <v>370</v>
       </c>
       <c r="N148" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O148" s="23" t="str">
         <f t="shared" si="2"/>
@@ -11990,7 +11990,7 @@
         <v>370</v>
       </c>
       <c r="N149" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O149" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12036,7 +12036,7 @@
         <v>277</v>
       </c>
       <c r="N150" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O150" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12080,7 +12080,7 @@
         <v>95</v>
       </c>
       <c r="N151" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O151" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12128,7 +12128,7 @@
         <v>394</v>
       </c>
       <c r="N152" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O152" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12176,7 +12176,7 @@
         <v>394</v>
       </c>
       <c r="N153" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O153" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12224,7 +12224,7 @@
         <v>822</v>
       </c>
       <c r="N154" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O154" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12270,7 +12270,7 @@
         <v>396</v>
       </c>
       <c r="N155" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O155" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12316,7 +12316,7 @@
         <v>396</v>
       </c>
       <c r="N156" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O156" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12362,7 +12362,7 @@
         <v>396</v>
       </c>
       <c r="N157" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O157" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12408,7 +12408,7 @@
         <v>207</v>
       </c>
       <c r="N158" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O158" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12454,7 +12454,7 @@
         <v>207</v>
       </c>
       <c r="N159" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O159" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12500,7 +12500,7 @@
         <v>207</v>
       </c>
       <c r="N160" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O160" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12546,7 +12546,7 @@
         <v>207</v>
       </c>
       <c r="N161" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O161" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12594,7 +12594,7 @@
         <v>103</v>
       </c>
       <c r="N162" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O162" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12642,14 +12642,14 @@
         <v>361</v>
       </c>
       <c r="N163" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O163" s="23" t="str">
         <f t="shared" si="2"/>
         <v>DATA/logos/M2C.png</v>
       </c>
     </row>
-    <row r="164" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>7</v>
       </c>
@@ -12684,7 +12684,7 @@
         <v>841</v>
       </c>
       <c r="N164" s="1" t="s">
-        <v>1440</v>
+        <v>1439</v>
       </c>
       <c r="O164" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12732,7 +12732,7 @@
         <v>372</v>
       </c>
       <c r="N165" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O165" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12780,7 +12780,7 @@
         <v>372</v>
       </c>
       <c r="N166" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O166" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12828,7 +12828,7 @@
         <v>372</v>
       </c>
       <c r="N167" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O167" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12876,7 +12876,7 @@
         <v>372</v>
       </c>
       <c r="N168" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O168" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12924,7 +12924,7 @@
         <v>285</v>
       </c>
       <c r="N169" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O169" s="23" t="str">
         <f t="shared" si="2"/>
@@ -12970,7 +12970,7 @@
         <v>398</v>
       </c>
       <c r="N170" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O170" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13016,7 +13016,7 @@
         <v>398</v>
       </c>
       <c r="N171" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O171" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13064,7 +13064,7 @@
         <v>297</v>
       </c>
       <c r="N172" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O172" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13112,7 +13112,7 @@
         <v>297</v>
       </c>
       <c r="N173" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O173" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13156,7 +13156,7 @@
         <v>859</v>
       </c>
       <c r="N174" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O174" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13204,7 +13204,7 @@
         <v>387</v>
       </c>
       <c r="N175" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O175" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13250,7 +13250,7 @@
         <v>60</v>
       </c>
       <c r="N176" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O176" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13296,7 +13296,7 @@
         <v>60</v>
       </c>
       <c r="N177" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O177" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13340,7 +13340,7 @@
         <v>870</v>
       </c>
       <c r="N178" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O178" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13386,7 +13386,7 @@
         <v>380</v>
       </c>
       <c r="N179" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O179" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13432,7 +13432,7 @@
         <v>380</v>
       </c>
       <c r="N180" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O180" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13480,7 +13480,7 @@
         <v>368</v>
       </c>
       <c r="N181" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O181" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13528,7 +13528,7 @@
         <v>368</v>
       </c>
       <c r="N182" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O182" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13576,7 +13576,7 @@
         <v>368</v>
       </c>
       <c r="N183" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O183" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13624,7 +13624,7 @@
         <v>19</v>
       </c>
       <c r="N184" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O184" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13672,7 +13672,7 @@
         <v>19</v>
       </c>
       <c r="N185" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O185" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13720,7 +13720,7 @@
         <v>19</v>
       </c>
       <c r="N186" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O186" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13766,7 +13766,7 @@
         <v>406</v>
       </c>
       <c r="N187" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O187" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13812,7 +13812,7 @@
         <v>406</v>
       </c>
       <c r="N188" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O188" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13856,7 +13856,7 @@
         <v>888</v>
       </c>
       <c r="N189" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O189" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13904,7 +13904,7 @@
         <v>288</v>
       </c>
       <c r="N190" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O190" s="23" t="str">
         <f t="shared" si="2"/>
@@ -13952,7 +13952,7 @@
         <v>408</v>
       </c>
       <c r="N191" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O191" s="23" t="str">
         <f t="shared" si="2"/>
@@ -14000,14 +14000,14 @@
         <v>411</v>
       </c>
       <c r="N192" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O192" s="23" t="str">
         <f t="shared" si="2"/>
         <v>DATA/logos/UMMISCO.png</v>
       </c>
     </row>
-    <row r="193" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A193" s="1" t="s">
         <v>7</v>
       </c>
@@ -14042,7 +14042,7 @@
         <v>905</v>
       </c>
       <c r="N193" s="1" t="s">
-        <v>1441</v>
+        <v>1440</v>
       </c>
       <c r="O193" s="23" t="str">
         <f t="shared" si="2"/>
@@ -14088,7 +14088,7 @@
         <v>344</v>
       </c>
       <c r="N194" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O194" s="23" t="str">
         <f t="shared" si="2"/>
@@ -14134,7 +14134,7 @@
         <v>389</v>
       </c>
       <c r="N195" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O195" s="23" t="str">
         <f t="shared" ref="O195:O258" si="3">"DATA/logos/" &amp; TEXT(E195,"jjj") &amp; ".png"</f>
@@ -14180,7 +14180,7 @@
         <v>389</v>
       </c>
       <c r="N196" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O196" s="23" t="str">
         <f t="shared" si="3"/>
@@ -14220,14 +14220,14 @@
         <v>915</v>
       </c>
       <c r="N197" s="1" t="s">
-        <v>1442</v>
+        <v>1441</v>
       </c>
       <c r="O197" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/CARDEC.png</v>
       </c>
     </row>
-    <row r="198" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>7</v>
       </c>
@@ -14262,7 +14262,7 @@
         <v>635</v>
       </c>
       <c r="N198" s="1" t="s">
-        <v>1437</v>
+        <v>1436</v>
       </c>
       <c r="O198" s="23" t="str">
         <f t="shared" si="3"/>
@@ -14308,7 +14308,7 @@
         <v>922</v>
       </c>
       <c r="N199" s="1" t="s">
-        <v>1443</v>
+        <v>1442</v>
       </c>
       <c r="O199" s="23" t="str">
         <f t="shared" si="3"/>
@@ -14348,7 +14348,7 @@
         <v>927</v>
       </c>
       <c r="N200" s="1" t="s">
-        <v>1444</v>
+        <v>1443</v>
       </c>
       <c r="O200" s="23" t="str">
         <f t="shared" si="3"/>
@@ -14396,7 +14396,7 @@
         <v>922</v>
       </c>
       <c r="N201" s="1" t="s">
-        <v>1443</v>
+        <v>1442</v>
       </c>
       <c r="O201" s="23" t="str">
         <f t="shared" si="3"/>
@@ -14434,14 +14434,14 @@
         <v>935</v>
       </c>
       <c r="N202" s="1" t="s">
-        <v>1445</v>
+        <v>1444</v>
       </c>
       <c r="O202" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/UZF.png</v>
       </c>
     </row>
-    <row r="203" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A203" s="1" t="s">
         <v>7</v>
       </c>
@@ -14470,14 +14470,14 @@
         <v>939</v>
       </c>
       <c r="N203" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O203" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac Leman.png</v>
       </c>
     </row>
-    <row r="204" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>7</v>
       </c>
@@ -14506,14 +14506,14 @@
         <v>942</v>
       </c>
       <c r="N204" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O204" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac Annecy.png</v>
       </c>
     </row>
-    <row r="205" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>7</v>
       </c>
@@ -14542,14 +14542,14 @@
         <v>945</v>
       </c>
       <c r="N205" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O205" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac Bourget.png</v>
       </c>
     </row>
-    <row r="206" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>7</v>
       </c>
@@ -14578,14 +14578,14 @@
         <v>948</v>
       </c>
       <c r="N206" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O206" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac Aiguebelette.png</v>
       </c>
     </row>
-    <row r="207" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>7</v>
       </c>
@@ -14614,14 +14614,14 @@
         <v>951</v>
       </c>
       <c r="N207" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O207" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac de Chavolet.png</v>
       </c>
     </row>
-    <row r="208" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>7</v>
       </c>
@@ -14650,14 +14650,14 @@
         <v>954</v>
       </c>
       <c r="N208" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O208" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac Pavin.png</v>
       </c>
     </row>
-    <row r="209" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>7</v>
       </c>
@@ -14686,14 +14686,14 @@
         <v>957</v>
       </c>
       <c r="N209" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O209" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac de Carcans Hourtin.png</v>
       </c>
     </row>
-    <row r="210" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>7</v>
       </c>
@@ -14722,14 +14722,14 @@
         <v>960</v>
       </c>
       <c r="N210" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O210" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac de Lacanau.png</v>
       </c>
     </row>
-    <row r="211" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
         <v>7</v>
       </c>
@@ -14758,14 +14758,14 @@
         <v>963</v>
       </c>
       <c r="N211" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O211" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac de Cazaux Sanguinet.png</v>
       </c>
     </row>
-    <row r="212" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A212" s="1" t="s">
         <v>7</v>
       </c>
@@ -14794,14 +14794,14 @@
         <v>966</v>
       </c>
       <c r="N212" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O212" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac de Parentis Biscarosse.png</v>
       </c>
     </row>
-    <row r="213" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>7</v>
       </c>
@@ -14830,14 +14830,14 @@
         <v>969</v>
       </c>
       <c r="N213" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O213" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Retenue de Serre Ponçon.png</v>
       </c>
     </row>
-    <row r="214" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>7</v>
       </c>
@@ -14866,14 +14866,14 @@
         <v>972</v>
       </c>
       <c r="N214" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O214" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Etang de Birieux.png</v>
       </c>
     </row>
-    <row r="215" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A215" s="1" t="s">
         <v>7</v>
       </c>
@@ -14902,14 +14902,14 @@
         <v>975</v>
       </c>
       <c r="N215" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O215" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Gravière Oselle.png</v>
       </c>
     </row>
-    <row r="216" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>7</v>
       </c>
@@ -14938,14 +14938,14 @@
         <v>978</v>
       </c>
       <c r="N216" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O216" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Reservoir de Charmes.png</v>
       </c>
     </row>
-    <row r="217" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>7</v>
       </c>
@@ -14974,14 +14974,14 @@
         <v>981</v>
       </c>
       <c r="N217" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O217" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Bernadouze.png</v>
       </c>
     </row>
-    <row r="218" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
         <v>7</v>
       </c>
@@ -15010,14 +15010,14 @@
         <v>984</v>
       </c>
       <c r="N218" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O218" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Frasnes.png</v>
       </c>
     </row>
-    <row r="219" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
         <v>7</v>
       </c>
@@ -15046,14 +15046,14 @@
         <v>987</v>
       </c>
       <c r="N219" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O219" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/La Guette.png</v>
       </c>
     </row>
-    <row r="220" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>7</v>
       </c>
@@ -15082,14 +15082,14 @@
         <v>990</v>
       </c>
       <c r="N220" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O220" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Puechabon.png</v>
       </c>
     </row>
-    <row r="221" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>7</v>
       </c>
@@ -15118,14 +15118,14 @@
         <v>993</v>
       </c>
       <c r="N221" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O221" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Font Blanche.png</v>
       </c>
     </row>
-    <row r="222" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>7</v>
       </c>
@@ -15154,14 +15154,14 @@
         <v>996</v>
       </c>
       <c r="N222" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O222" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Bilos.png</v>
       </c>
     </row>
-    <row r="223" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>7</v>
       </c>
@@ -15190,14 +15190,14 @@
         <v>999</v>
       </c>
       <c r="N223" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O223" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Barbeau.png</v>
       </c>
     </row>
-    <row r="224" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>7</v>
       </c>
@@ -15226,14 +15226,14 @@
         <v>1002</v>
       </c>
       <c r="N224" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O224" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Hesse.png</v>
       </c>
     </row>
-    <row r="225" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>7</v>
       </c>
@@ -15262,14 +15262,14 @@
         <v>1005</v>
       </c>
       <c r="N225" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O225" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/O3HP.png</v>
       </c>
     </row>
-    <row r="226" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>7</v>
       </c>
@@ -15298,14 +15298,14 @@
         <v>1008</v>
       </c>
       <c r="N226" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O226" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Montiers.png</v>
       </c>
     </row>
-    <row r="227" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>7</v>
       </c>
@@ -15339,7 +15339,7 @@
         <v>DATA/logos/Itatinga.png</v>
       </c>
     </row>
-    <row r="228" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>7</v>
       </c>
@@ -15368,14 +15368,14 @@
         <v>1014</v>
       </c>
       <c r="N228" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O228" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Estrees Mons.png</v>
       </c>
     </row>
-    <row r="229" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>7</v>
       </c>
@@ -15404,14 +15404,14 @@
         <v>1017</v>
       </c>
       <c r="N229" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O229" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Epoisses.png</v>
       </c>
     </row>
-    <row r="230" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>7</v>
       </c>
@@ -15440,14 +15440,14 @@
         <v>1020</v>
       </c>
       <c r="N230" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O230" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Auzeville.png</v>
       </c>
     </row>
-    <row r="231" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>7</v>
       </c>
@@ -15476,14 +15476,14 @@
         <v>1023</v>
       </c>
       <c r="N231" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O231" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Mauguio.png</v>
       </c>
     </row>
-    <row r="232" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>7</v>
       </c>
@@ -15517,7 +15517,7 @@
         <v>DATA/logos/Bac Giang.png</v>
       </c>
     </row>
-    <row r="233" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>7</v>
       </c>
@@ -15551,7 +15551,7 @@
         <v>DATA/logos/Battambang.png</v>
       </c>
     </row>
-    <row r="234" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A234" s="1" t="s">
         <v>7</v>
       </c>
@@ -15585,7 +15585,7 @@
         <v>DATA/logos/Bos khnor.png</v>
       </c>
     </row>
-    <row r="235" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A235" s="1" t="s">
         <v>7</v>
       </c>
@@ -15619,7 +15619,7 @@
         <v>DATA/logos/Harare.png</v>
       </c>
     </row>
-    <row r="236" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A236" s="1" t="s">
         <v>7</v>
       </c>
@@ -15648,14 +15648,14 @@
         <v>990</v>
       </c>
       <c r="N236" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O236" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Puechabon.png</v>
       </c>
     </row>
-    <row r="237" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A237" s="1" t="s">
         <v>7</v>
       </c>
@@ -15684,14 +15684,14 @@
         <v>993</v>
       </c>
       <c r="N237" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O237" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Font Blanche.png</v>
       </c>
     </row>
-    <row r="238" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A238" s="1" t="s">
         <v>7</v>
       </c>
@@ -15720,14 +15720,14 @@
         <v>1005</v>
       </c>
       <c r="N238" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O238" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/O3HP.png</v>
       </c>
     </row>
-    <row r="239" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A239" s="1" t="s">
         <v>7</v>
       </c>
@@ -15756,14 +15756,14 @@
         <v>1008</v>
       </c>
       <c r="N239" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O239" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Montiers.png</v>
       </c>
     </row>
-    <row r="240" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
         <v>7</v>
       </c>
@@ -15792,14 +15792,14 @@
         <v>939</v>
       </c>
       <c r="N240" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O240" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac Leman.png</v>
       </c>
     </row>
-    <row r="241" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
         <v>7</v>
       </c>
@@ -15828,14 +15828,14 @@
         <v>942</v>
       </c>
       <c r="N241" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O241" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac Annecy.png</v>
       </c>
     </row>
-    <row r="242" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>7</v>
       </c>
@@ -15864,14 +15864,14 @@
         <v>945</v>
       </c>
       <c r="N242" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O242" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac Bourget.png</v>
       </c>
     </row>
-    <row r="243" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>7</v>
       </c>
@@ -15900,14 +15900,14 @@
         <v>948</v>
       </c>
       <c r="N243" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O243" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac Aiguebelette.png</v>
       </c>
     </row>
-    <row r="244" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>7</v>
       </c>
@@ -15936,14 +15936,14 @@
         <v>951</v>
       </c>
       <c r="N244" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O244" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lac de Chavolet.png</v>
       </c>
     </row>
-    <row r="245" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
         <v>7</v>
       </c>
@@ -15972,14 +15972,14 @@
         <v>972</v>
       </c>
       <c r="N245" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O245" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Etang de Birieux.png</v>
       </c>
     </row>
-    <row r="246" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
         <v>7</v>
       </c>
@@ -16008,14 +16008,14 @@
         <v>978</v>
       </c>
       <c r="N246" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O246" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Reservoir de Charmes.png</v>
       </c>
     </row>
-    <row r="247" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>7</v>
       </c>
@@ -16044,14 +16044,14 @@
         <v>1014</v>
       </c>
       <c r="N247" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O247" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Estrees Mons.png</v>
       </c>
     </row>
-    <row r="248" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>7</v>
       </c>
@@ -16080,14 +16080,14 @@
         <v>1038</v>
       </c>
       <c r="N248" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O248" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Feucherolles.png</v>
       </c>
     </row>
-    <row r="249" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>7</v>
       </c>
@@ -16116,14 +16116,14 @@
         <v>1017</v>
       </c>
       <c r="N249" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O249" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Epoisses.png</v>
       </c>
     </row>
-    <row r="250" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
         <v>7</v>
       </c>
@@ -16152,14 +16152,14 @@
         <v>1041</v>
       </c>
       <c r="N250" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O250" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Lusignan.png</v>
       </c>
     </row>
-    <row r="251" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
         <v>7</v>
       </c>
@@ -16188,14 +16188,14 @@
         <v>1044</v>
       </c>
       <c r="N251" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O251" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Theix.png</v>
       </c>
     </row>
-    <row r="252" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
         <v>7</v>
       </c>
@@ -16224,14 +16224,14 @@
         <v>1047</v>
       </c>
       <c r="N252" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O252" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Laqueille.png</v>
       </c>
     </row>
-    <row r="253" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
         <v>7</v>
       </c>
@@ -16260,14 +16260,14 @@
         <v>1050</v>
       </c>
       <c r="N253" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O253" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/La Bouzule.png</v>
       </c>
     </row>
-    <row r="254" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
         <v>7</v>
       </c>
@@ -16296,14 +16296,14 @@
         <v>1053</v>
       </c>
       <c r="N254" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O254" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/Breuil chenue.png</v>
       </c>
     </row>
-    <row r="255" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
         <v>7</v>
       </c>
@@ -16337,7 +16337,7 @@
         <v>DATA/logos/Couanimi.png</v>
       </c>
     </row>
-    <row r="256" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
         <v>7</v>
       </c>
@@ -16371,7 +16371,7 @@
         <v>DATA/logos/Crique Plomb.png</v>
       </c>
     </row>
-    <row r="257" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A257" s="1" t="s">
         <v>7</v>
       </c>
@@ -16405,7 +16405,7 @@
         <v>DATA/logos/Paracou.png</v>
       </c>
     </row>
-    <row r="258" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
         <v>7</v>
       </c>
@@ -16439,7 +16439,7 @@
         <v>DATA/logos/Belefoungu.png</v>
       </c>
     </row>
-    <row r="259" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
         <v>7</v>
       </c>
@@ -16473,7 +16473,7 @@
         <v>DATA/logos/Mata flux.png</v>
       </c>
     </row>
-    <row r="260" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
         <v>7</v>
       </c>
@@ -16507,7 +16507,7 @@
         <v>DATA/logos/Cacao flux.png</v>
       </c>
     </row>
-    <row r="261" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
         <v>7</v>
       </c>
@@ -16541,7 +16541,7 @@
         <v>DATA/logos/Carpaag.png</v>
       </c>
     </row>
-    <row r="262" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
         <v>7</v>
       </c>
@@ -16575,7 +16575,7 @@
         <v>DATA/logos/Mule Hole.png</v>
       </c>
     </row>
-    <row r="263" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A263" s="1" t="s">
         <v>7</v>
       </c>
@@ -16609,7 +16609,7 @@
         <v>DATA/logos/Tensift.png</v>
       </c>
     </row>
-    <row r="264" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
         <v>7</v>
       </c>
@@ -16643,7 +16643,7 @@
         <v>DATA/logos/Wankama.png</v>
       </c>
     </row>
-    <row r="265" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
         <v>7</v>
       </c>
@@ -16677,7 +16677,7 @@
         <v>DATA/logos/Niakhar.png</v>
       </c>
     </row>
-    <row r="266" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
         <v>7</v>
       </c>
@@ -16711,7 +16711,7 @@
         <v>DATA/logos/Niakhar sob.png</v>
       </c>
     </row>
-    <row r="267" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
         <v>7</v>
       </c>
@@ -16745,7 +16745,7 @@
         <v>DATA/logos/Niakhar ragola.png</v>
       </c>
     </row>
-    <row r="268" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
         <v>7</v>
       </c>
@@ -16779,7 +16779,7 @@
         <v>DATA/logos/Kamech.png</v>
       </c>
     </row>
-    <row r="269" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
         <v>7</v>
       </c>
@@ -16842,14 +16842,14 @@
         <v>1097</v>
       </c>
       <c r="N270" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O270" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Bassin versant du Couesnon.png</v>
       </c>
     </row>
-    <row r="271" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
         <v>7</v>
       </c>
@@ -16878,7 +16878,7 @@
         <v>1100</v>
       </c>
       <c r="N271" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O271" s="23" t="str">
         <f t="shared" si="4"/>
@@ -16914,14 +16914,14 @@
         <v>1103</v>
       </c>
       <c r="N272" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O272" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/bassin de la Doller et Déodatie.png</v>
       </c>
     </row>
-    <row r="273" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A273" s="1" t="s">
         <v>7</v>
       </c>
@@ -16950,14 +16950,14 @@
         <v>1106</v>
       </c>
       <c r="N273" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O273" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Ouvèze Ventoux.png</v>
       </c>
     </row>
-    <row r="274" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A274" s="1" t="s">
         <v>7</v>
       </c>
@@ -16991,7 +16991,7 @@
         <v>DATA/logos/Ile de la Reunion.png</v>
       </c>
     </row>
-    <row r="275" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A275" s="1" t="s">
         <v>7</v>
       </c>
@@ -17025,7 +17025,7 @@
         <v>DATA/logos/Bassin versant du Ferlo.png</v>
       </c>
     </row>
-    <row r="276" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A276" s="1" t="s">
         <v>7</v>
       </c>
@@ -17059,7 +17059,7 @@
         <v>DATA/logos/Guadeloupe.png</v>
       </c>
     </row>
-    <row r="277" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A277" s="1" t="s">
         <v>7</v>
       </c>
@@ -17088,14 +17088,14 @@
         <v>1118</v>
       </c>
       <c r="N277" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O277" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Pierroton Xylosylve.png</v>
       </c>
     </row>
-    <row r="278" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A278" s="1" t="s">
         <v>7</v>
       </c>
@@ -17129,7 +17129,7 @@
         <v>DATA/logos/Itatinga.png</v>
       </c>
     </row>
-    <row r="279" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A279" s="1" t="s">
         <v>7</v>
       </c>
@@ -17158,14 +17158,14 @@
         <v>999</v>
       </c>
       <c r="N279" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O279" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Barbeau.png</v>
       </c>
     </row>
-    <row r="280" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A280" s="1" t="s">
         <v>7</v>
       </c>
@@ -17194,14 +17194,14 @@
         <v>996</v>
       </c>
       <c r="N280" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O280" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Bilos.png</v>
       </c>
     </row>
-    <row r="281" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A281" s="1" t="s">
         <v>7</v>
       </c>
@@ -17230,14 +17230,14 @@
         <v>1002</v>
       </c>
       <c r="N281" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O281" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Hesse.png</v>
       </c>
     </row>
-    <row r="282" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A282" s="1" t="s">
         <v>7</v>
       </c>
@@ -17271,7 +17271,7 @@
         <v>DATA/logos/Abisko.png</v>
       </c>
     </row>
-    <row r="283" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>7</v>
       </c>
@@ -17305,7 +17305,7 @@
         <v>DATA/logos/Zackenberg.png</v>
       </c>
     </row>
-    <row r="284" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A284" s="1" t="s">
         <v>7</v>
       </c>
@@ -17339,7 +17339,7 @@
         <v>DATA/logos/Churchill.png</v>
       </c>
     </row>
-    <row r="285" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A285" s="1" t="s">
         <v>7</v>
       </c>
@@ -17373,7 +17373,7 @@
         <v>DATA/logos/Manche a eau.png</v>
       </c>
     </row>
-    <row r="286" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>7</v>
       </c>
@@ -17407,7 +17407,7 @@
         <v>DATA/logos/La Lezarde.png</v>
       </c>
     </row>
-    <row r="287" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A287" s="1" t="s">
         <v>7</v>
       </c>
@@ -17441,7 +17441,7 @@
         <v>DATA/logos/Cayenne.png</v>
       </c>
     </row>
-    <row r="288" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
         <v>7</v>
       </c>
@@ -17475,7 +17475,7 @@
         <v>DATA/logos/Crique Fouille.png</v>
       </c>
     </row>
-    <row r="289" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A289" s="1" t="s">
         <v>7</v>
       </c>
@@ -17509,7 +17509,7 @@
         <v>DATA/logos/Mahury.png</v>
       </c>
     </row>
-    <row r="290" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A290" s="1" t="s">
         <v>7</v>
       </c>
@@ -17543,7 +17543,7 @@
         <v>DATA/logos/Mamangua.png</v>
       </c>
     </row>
-    <row r="291" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A291" s="1" t="s">
         <v>7</v>
       </c>
@@ -17577,7 +17577,7 @@
         <v>DATA/logos/Guaratiba.png</v>
       </c>
     </row>
-    <row r="292" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A292" s="1" t="s">
         <v>7</v>
       </c>
@@ -17611,7 +17611,7 @@
         <v>DATA/logos/Marapanim.png</v>
       </c>
     </row>
-    <row r="293" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A293" s="1" t="s">
         <v>7</v>
       </c>
@@ -17645,7 +17645,7 @@
         <v>DATA/logos/Can Gio.png</v>
       </c>
     </row>
-    <row r="294" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
         <v>7</v>
       </c>
@@ -17679,7 +17679,7 @@
         <v>DATA/logos/Ouvea.png</v>
       </c>
     </row>
-    <row r="295" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
         <v>7</v>
       </c>
@@ -17713,7 +17713,7 @@
         <v>DATA/logos/Dumbea.png</v>
       </c>
     </row>
-    <row r="296" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
         <v>7</v>
       </c>
@@ -17742,14 +17742,14 @@
         <v>1162</v>
       </c>
       <c r="N296" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O296" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Bassin Arcachon.png</v>
       </c>
     </row>
-    <row r="297" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
         <v>7</v>
       </c>
@@ -17778,14 +17778,14 @@
         <v>1165</v>
       </c>
       <c r="N297" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O297" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Mortagne-sur-Gironde.png</v>
       </c>
     </row>
-    <row r="298" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
         <v>7</v>
       </c>
@@ -17814,14 +17814,14 @@
         <v>1168</v>
       </c>
       <c r="N298" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O298" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Littoral charentais.png</v>
       </c>
     </row>
-    <row r="299" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>7</v>
       </c>
@@ -17850,14 +17850,14 @@
         <v>1171</v>
       </c>
       <c r="N299" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O299" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Estuaire de la Loire.png</v>
       </c>
     </row>
-    <row r="300" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
         <v>7</v>
       </c>
@@ -17886,14 +17886,14 @@
         <v>1174</v>
       </c>
       <c r="N300" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O300" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Rade de Brest.png</v>
       </c>
     </row>
-    <row r="301" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
         <v>7</v>
       </c>
@@ -17922,14 +17922,14 @@
         <v>1177</v>
       </c>
       <c r="N301" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O301" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Estuaire du Trieux.png</v>
       </c>
     </row>
-    <row r="302" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>7</v>
       </c>
@@ -17958,14 +17958,14 @@
         <v>1180</v>
       </c>
       <c r="N302" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O302" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Anse du Cul-de-Loup.png</v>
       </c>
     </row>
-    <row r="303" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>7</v>
       </c>
@@ -17994,14 +17994,14 @@
         <v>1183</v>
       </c>
       <c r="N303" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O303" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Baie de Bourgneuf.png</v>
       </c>
     </row>
-    <row r="304" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
         <v>7</v>
       </c>
@@ -18030,14 +18030,14 @@
         <v>1186</v>
       </c>
       <c r="N304" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O304" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Estuaire de la Canche.png</v>
       </c>
     </row>
-    <row r="305" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
         <v>7</v>
       </c>
@@ -18066,14 +18066,14 @@
         <v>1189</v>
       </c>
       <c r="N305" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O305" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de Clairvaux.png</v>
       </c>
     </row>
-    <row r="306" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>7</v>
       </c>
@@ -18102,14 +18102,14 @@
         <v>1192</v>
       </c>
       <c r="N306" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O306" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de Maclu.png</v>
       </c>
     </row>
-    <row r="307" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>7</v>
       </c>
@@ -18138,14 +18138,14 @@
         <v>1195</v>
       </c>
       <c r="N307" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O307" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de Petit Maclu.png</v>
       </c>
     </row>
-    <row r="308" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>7</v>
       </c>
@@ -18174,14 +18174,14 @@
         <v>1198</v>
       </c>
       <c r="N308" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O308" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de Chalain.png</v>
       </c>
     </row>
-    <row r="309" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>7</v>
       </c>
@@ -18210,14 +18210,14 @@
         <v>1201</v>
       </c>
       <c r="N309" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O309" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac d'Ilay.png</v>
       </c>
     </row>
-    <row r="310" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
         <v>7</v>
       </c>
@@ -18246,14 +18246,14 @@
         <v>1204</v>
       </c>
       <c r="N310" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O310" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de Narlay.png</v>
       </c>
     </row>
-    <row r="311" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
         <v>7</v>
       </c>
@@ -18282,14 +18282,14 @@
         <v>1207</v>
       </c>
       <c r="N311" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O311" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de Remoray.png</v>
       </c>
     </row>
-    <row r="312" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A312" s="1" t="s">
         <v>7</v>
       </c>
@@ -18318,14 +18318,14 @@
         <v>1210</v>
       </c>
       <c r="N312" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O312" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de Saint Point.png</v>
       </c>
     </row>
-    <row r="313" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A313" s="1" t="s">
         <v>7</v>
       </c>
@@ -18354,14 +18354,14 @@
         <v>1213</v>
       </c>
       <c r="N313" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O313" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de Bonlieu.png</v>
       </c>
     </row>
-    <row r="314" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
         <v>7</v>
       </c>
@@ -18390,14 +18390,14 @@
         <v>1216</v>
       </c>
       <c r="N314" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O314" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de l'Abbaye.png</v>
       </c>
     </row>
-    <row r="315" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
         <v>7</v>
       </c>
@@ -18426,14 +18426,14 @@
         <v>1219</v>
       </c>
       <c r="N315" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O315" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de Nantua.png</v>
       </c>
     </row>
-    <row r="316" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A316" s="1" t="s">
         <v>7</v>
       </c>
@@ -18462,14 +18462,14 @@
         <v>1222</v>
       </c>
       <c r="N316" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O316" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac des Rousses.png</v>
       </c>
     </row>
-    <row r="317" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A317" s="1" t="s">
         <v>7</v>
       </c>
@@ -18498,14 +18498,14 @@
         <v>1225</v>
       </c>
       <c r="N317" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O317" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de Bellefontaine.png</v>
       </c>
     </row>
-    <row r="318" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
         <v>7</v>
       </c>
@@ -18534,14 +18534,14 @@
         <v>1228</v>
       </c>
       <c r="N318" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O318" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac des Mortes.png</v>
       </c>
     </row>
-    <row r="319" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
         <v>7</v>
       </c>
@@ -18570,14 +18570,14 @@
         <v>1231</v>
       </c>
       <c r="N319" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O319" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Etang du Pont rouge.png</v>
       </c>
     </row>
-    <row r="320" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
         <v>7</v>
       </c>
@@ -18606,14 +18606,14 @@
         <v>1234</v>
       </c>
       <c r="N320" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O320" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de Gerardmer.png</v>
       </c>
     </row>
-    <row r="321" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
         <v>7</v>
       </c>
@@ -18642,14 +18642,14 @@
         <v>1237</v>
       </c>
       <c r="N321" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O321" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de Longemer.png</v>
       </c>
     </row>
-    <row r="322" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
         <v>7</v>
       </c>
@@ -18678,14 +18678,14 @@
         <v>1240</v>
       </c>
       <c r="N322" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O322" s="23" t="str">
         <f t="shared" si="4"/>
         <v>DATA/logos/Lac de la Maix.png</v>
       </c>
     </row>
-    <row r="323" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>7</v>
       </c>
@@ -18714,14 +18714,14 @@
         <v>1243</v>
       </c>
       <c r="N323" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O323" s="23" t="str">
         <f t="shared" ref="O323:O386" si="5">"DATA/logos/" &amp; TEXT(E323,"jjj") &amp; ".png"</f>
         <v>DATA/logos/Lac des Corbeaux.png</v>
       </c>
     </row>
-    <row r="324" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>7</v>
       </c>
@@ -18750,14 +18750,14 @@
         <v>1246</v>
       </c>
       <c r="N324" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O324" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de Blanchemer.png</v>
       </c>
     </row>
-    <row r="325" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
         <v>7</v>
       </c>
@@ -18786,14 +18786,14 @@
         <v>1249</v>
       </c>
       <c r="N325" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O325" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac Marion.png</v>
       </c>
     </row>
-    <row r="326" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>7</v>
       </c>
@@ -18822,14 +18822,14 @@
         <v>1252</v>
       </c>
       <c r="N326" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O326" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac Mourisot.png</v>
       </c>
     </row>
-    <row r="327" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>7</v>
       </c>
@@ -18858,14 +18858,14 @@
         <v>1255</v>
       </c>
       <c r="N327" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O327" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Wildsee.png</v>
       </c>
     </row>
-    <row r="328" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A328" s="1" t="s">
         <v>7</v>
       </c>
@@ -18894,14 +18894,14 @@
         <v>1258</v>
       </c>
       <c r="N328" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O328" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de la Godivelle.png</v>
       </c>
     </row>
-    <row r="329" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A329" s="1" t="s">
         <v>7</v>
       </c>
@@ -18930,14 +18930,14 @@
         <v>1261</v>
       </c>
       <c r="N329" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O329" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de la Landie.png</v>
       </c>
     </row>
-    <row r="330" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A330" s="1" t="s">
         <v>7</v>
       </c>
@@ -18966,14 +18966,14 @@
         <v>1264</v>
       </c>
       <c r="N330" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O330" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de Montcineyre.png</v>
       </c>
     </row>
-    <row r="331" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A331" s="1" t="s">
         <v>7</v>
       </c>
@@ -19002,14 +19002,14 @@
         <v>1267</v>
       </c>
       <c r="N331" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O331" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de Guery.png</v>
       </c>
     </row>
-    <row r="332" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A332" s="1" t="s">
         <v>7</v>
       </c>
@@ -19038,14 +19038,14 @@
         <v>1270</v>
       </c>
       <c r="N332" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O332" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac Verdet.png</v>
       </c>
     </row>
-    <row r="333" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A333" s="1" t="s">
         <v>7</v>
       </c>
@@ -19074,14 +19074,14 @@
         <v>1273</v>
       </c>
       <c r="N333" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O333" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac du Mont-Coua.png</v>
       </c>
     </row>
-    <row r="334" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
         <v>7</v>
       </c>
@@ -19110,14 +19110,14 @@
         <v>1276</v>
       </c>
       <c r="N334" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O334" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac du Brévent.png</v>
       </c>
     </row>
-    <row r="335" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
         <v>7</v>
       </c>
@@ -19146,14 +19146,14 @@
         <v>1279</v>
       </c>
       <c r="N335" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O335" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de Paladru.png</v>
       </c>
     </row>
-    <row r="336" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A336" s="1" t="s">
         <v>7</v>
       </c>
@@ -19182,14 +19182,14 @@
         <v>1281</v>
       </c>
       <c r="N336" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O336" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac d'Anterne.png</v>
       </c>
     </row>
-    <row r="337" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A337" s="1" t="s">
         <v>7</v>
       </c>
@@ -19218,14 +19218,14 @@
         <v>1283</v>
       </c>
       <c r="N337" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O337" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac d'Allos.png</v>
       </c>
     </row>
-    <row r="338" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A338" s="1" t="s">
         <v>7</v>
       </c>
@@ -19254,14 +19254,14 @@
         <v>1286</v>
       </c>
       <c r="N338" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O338" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac du Lauzanier.png</v>
       </c>
     </row>
-    <row r="339" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A339" s="1" t="s">
         <v>7</v>
       </c>
@@ -19290,14 +19290,14 @@
         <v>1289</v>
       </c>
       <c r="N339" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O339" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de la Thuile.png</v>
       </c>
     </row>
-    <row r="340" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A340" s="1" t="s">
         <v>7</v>
       </c>
@@ -19326,14 +19326,14 @@
         <v>1292</v>
       </c>
       <c r="N340" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O340" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac Blanc (Aiguilles rouges).png</v>
       </c>
     </row>
-    <row r="341" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A341" s="1" t="s">
         <v>7</v>
       </c>
@@ -19362,14 +19362,14 @@
         <v>1295</v>
       </c>
       <c r="N341" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O341" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac Bénit.png</v>
       </c>
     </row>
-    <row r="342" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A342" s="1" t="s">
         <v>7</v>
       </c>
@@ -19398,14 +19398,14 @@
         <v>1298</v>
       </c>
       <c r="N342" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O342" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de Gers.png</v>
       </c>
     </row>
-    <row r="343" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A343" s="1" t="s">
         <v>7</v>
       </c>
@@ -19434,14 +19434,14 @@
         <v>1301</v>
       </c>
       <c r="N343" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O343" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de la Muzelle.png</v>
       </c>
     </row>
-    <row r="344" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A344" s="1" t="s">
         <v>7</v>
       </c>
@@ -19470,14 +19470,14 @@
         <v>1304</v>
       </c>
       <c r="N344" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O344" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac du Lauvitel.png</v>
       </c>
     </row>
-    <row r="345" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A345" s="1" t="s">
         <v>7</v>
       </c>
@@ -19506,14 +19506,14 @@
         <v>1307</v>
       </c>
       <c r="N345" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O345" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac Robert.png</v>
       </c>
     </row>
-    <row r="346" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A346" s="1" t="s">
         <v>7</v>
       </c>
@@ -19542,14 +19542,14 @@
         <v>1310</v>
       </c>
       <c r="N346" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O346" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de Bastani.png</v>
       </c>
     </row>
-    <row r="347" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A347" s="1" t="s">
         <v>7</v>
       </c>
@@ -19578,14 +19578,14 @@
         <v>1313</v>
       </c>
       <c r="N347" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O347" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de Nino.png</v>
       </c>
     </row>
-    <row r="348" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A348" s="1" t="s">
         <v>7</v>
       </c>
@@ -19614,14 +19614,14 @@
         <v>1316</v>
       </c>
       <c r="N348" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O348" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Etang d'Urbino.png</v>
       </c>
     </row>
-    <row r="349" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A349" s="1" t="s">
         <v>7</v>
       </c>
@@ -19650,14 +19650,14 @@
         <v>1319</v>
       </c>
       <c r="N349" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O349" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de Mélo.png</v>
       </c>
     </row>
-    <row r="350" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A350" s="1" t="s">
         <v>7</v>
       </c>
@@ -19686,14 +19686,14 @@
         <v>1322</v>
       </c>
       <c r="N350" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O350" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de Capitello.png</v>
       </c>
     </row>
-    <row r="351" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A351" s="1" t="s">
         <v>7</v>
       </c>
@@ -19722,14 +19722,14 @@
         <v>1325</v>
       </c>
       <c r="N351" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O351" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac Nègre.png</v>
       </c>
     </row>
-    <row r="352" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A352" s="1" t="s">
         <v>7</v>
       </c>
@@ -19758,14 +19758,14 @@
         <v>1328</v>
       </c>
       <c r="N352" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O352" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Grand Lac.png</v>
       </c>
     </row>
-    <row r="353" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A353" s="1" t="s">
         <v>7</v>
       </c>
@@ -19794,14 +19794,14 @@
         <v>1331</v>
       </c>
       <c r="N353" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O353" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de la Ponssonière.png</v>
       </c>
     </row>
-    <row r="354" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A354" s="1" t="s">
         <v>7</v>
       </c>
@@ -19830,14 +19830,14 @@
         <v>1334</v>
       </c>
       <c r="N354" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O354" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de l'Eychauda.png</v>
       </c>
     </row>
-    <row r="355" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A355" s="1" t="s">
         <v>7</v>
       </c>
@@ -19866,14 +19866,14 @@
         <v>1337</v>
       </c>
       <c r="N355" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O355" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de Tignes.png</v>
       </c>
     </row>
-    <row r="356" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A356" s="1" t="s">
         <v>7</v>
       </c>
@@ -19902,14 +19902,14 @@
         <v>1340</v>
       </c>
       <c r="N356" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O356" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de Plan Vianney.png</v>
       </c>
     </row>
-    <row r="357" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A357" s="1" t="s">
         <v>7</v>
       </c>
@@ -19938,14 +19938,14 @@
         <v>1343</v>
       </c>
       <c r="N357" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O357" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac du Verney.png</v>
       </c>
     </row>
-    <row r="358" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A358" s="1" t="s">
         <v>7</v>
       </c>
@@ -19974,14 +19974,14 @@
         <v>1346</v>
       </c>
       <c r="N358" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O358" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac Luitel.png</v>
       </c>
     </row>
-    <row r="359" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A359" s="1" t="s">
         <v>7</v>
       </c>
@@ -20010,14 +20010,14 @@
         <v>1349</v>
       </c>
       <c r="N359" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O359" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac d'Arvouin.png</v>
       </c>
     </row>
-    <row r="360" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A360" s="1" t="s">
         <v>7</v>
       </c>
@@ -20046,14 +20046,14 @@
         <v>1352</v>
       </c>
       <c r="N360" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O360" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac du Loup.png</v>
       </c>
     </row>
-    <row r="361" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A361" s="1" t="s">
         <v>7</v>
       </c>
@@ -20082,14 +20082,14 @@
         <v>1355</v>
       </c>
       <c r="N361" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O361" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de la Plagne.png</v>
       </c>
     </row>
-    <row r="362" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A362" s="1" t="s">
         <v>7</v>
       </c>
@@ -20118,14 +20118,14 @@
         <v>1358</v>
       </c>
       <c r="N362" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O362" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de Saint André.png</v>
       </c>
     </row>
-    <row r="363" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A363" s="1" t="s">
         <v>7</v>
       </c>
@@ -20154,14 +20154,14 @@
         <v>1361</v>
       </c>
       <c r="N363" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O363" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac Savines.png</v>
       </c>
     </row>
-    <row r="364" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A364" s="1" t="s">
         <v>7</v>
       </c>
@@ -20190,14 +20190,14 @@
         <v>1364</v>
       </c>
       <c r="N364" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O364" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac du Doménon.png</v>
       </c>
     </row>
-    <row r="365" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A365" s="1" t="s">
         <v>7</v>
       </c>
@@ -20226,14 +20226,14 @@
         <v>1367</v>
       </c>
       <c r="N365" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O365" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lacs de la Braissette.png</v>
       </c>
     </row>
-    <row r="366" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A366" s="1" t="s">
         <v>7</v>
       </c>
@@ -20262,14 +20262,14 @@
         <v>1370</v>
       </c>
       <c r="N366" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O366" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lagune Pierre Blanche.png</v>
       </c>
     </row>
-    <row r="367" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A367" s="1" t="s">
         <v>7</v>
       </c>
@@ -20298,14 +20298,14 @@
         <v>1373</v>
       </c>
       <c r="N367" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O367" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Etang de Lannenec.png</v>
       </c>
     </row>
-    <row r="368" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A368" s="1" t="s">
         <v>7</v>
       </c>
@@ -20334,14 +20334,14 @@
         <v>1376</v>
       </c>
       <c r="N368" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O368" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Etang de la Beulie.png</v>
       </c>
     </row>
-    <row r="369" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A369" s="1" t="s">
         <v>7</v>
       </c>
@@ -20370,14 +20370,14 @@
         <v>1379</v>
       </c>
       <c r="N369" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O369" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Estany Gros.png</v>
       </c>
     </row>
-    <row r="370" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A370" s="1" t="s">
         <v>7</v>
       </c>
@@ -20406,14 +20406,14 @@
         <v>1382</v>
       </c>
       <c r="N370" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O370" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Estany del Mig.png</v>
       </c>
     </row>
-    <row r="371" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A371" s="1" t="s">
         <v>7</v>
       </c>
@@ -20442,14 +20442,14 @@
         <v>1385</v>
       </c>
       <c r="N371" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O371" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac d'Espingo.png</v>
       </c>
     </row>
-    <row r="372" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A372" s="1" t="s">
         <v>7</v>
       </c>
@@ -20478,14 +20478,14 @@
         <v>1388</v>
       </c>
       <c r="N372" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O372" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac Gentau.png</v>
       </c>
     </row>
-    <row r="373" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A373" s="1" t="s">
         <v>7</v>
       </c>
@@ -20514,7 +20514,7 @@
         <v>1391</v>
       </c>
       <c r="N373" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O373" s="23" t="str">
         <f t="shared" si="5"/>
@@ -20550,14 +20550,14 @@
         <v>1394</v>
       </c>
       <c r="N374" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O374" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Etang de Sarrat de Montestaure.png</v>
       </c>
     </row>
-    <row r="375" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A375" s="1" t="s">
         <v>7</v>
       </c>
@@ -20586,14 +20586,14 @@
         <v>1397</v>
       </c>
       <c r="N375" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O375" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Etang de la Soucaranne.png</v>
       </c>
     </row>
-    <row r="376" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A376" s="1" t="s">
         <v>7</v>
       </c>
@@ -20622,14 +20622,14 @@
         <v>1400</v>
       </c>
       <c r="N376" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O376" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lac de Barroude.png</v>
       </c>
     </row>
-    <row r="377" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A377" s="1" t="s">
         <v>7</v>
       </c>
@@ -20658,14 +20658,14 @@
         <v>1403</v>
       </c>
       <c r="N377" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O377" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Etang de Sigriou.png</v>
       </c>
     </row>
-    <row r="378" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A378" s="1" t="s">
         <v>7</v>
       </c>
@@ -20694,14 +20694,14 @@
         <v>1406</v>
       </c>
       <c r="N378" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O378" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Villiers-le-Bâcle.png</v>
       </c>
     </row>
-    <row r="379" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A379" s="1" t="s">
         <v>7</v>
       </c>
@@ -20730,14 +20730,14 @@
         <v>1409</v>
       </c>
       <c r="N379" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O379" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Greoux.png</v>
       </c>
     </row>
-    <row r="380" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A380" s="1" t="s">
         <v>7</v>
       </c>
@@ -20766,14 +20766,14 @@
         <v>1412</v>
       </c>
       <c r="N380" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O380" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Lagon Arcachon.png</v>
       </c>
     </row>
-    <row r="381" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A381" s="1" t="s">
         <v>7</v>
       </c>
@@ -20802,14 +20802,14 @@
         <v>1415</v>
       </c>
       <c r="N381" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O381" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Seudre.png</v>
       </c>
     </row>
-    <row r="382" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A382" s="1" t="s">
         <v>7</v>
       </c>
@@ -20838,14 +20838,14 @@
         <v>1417</v>
       </c>
       <c r="N382" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O382" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Estuaire de la Loire.png</v>
       </c>
     </row>
-    <row r="383" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A383" s="1" t="s">
         <v>7</v>
       </c>
@@ -20874,14 +20874,14 @@
         <v>1419</v>
       </c>
       <c r="N383" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O383" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Baie de Bourgneuf.png</v>
       </c>
     </row>
-    <row r="384" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A384" s="1" t="s">
         <v>7</v>
       </c>
@@ -20910,14 +20910,14 @@
         <v>1421</v>
       </c>
       <c r="N384" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O384" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Rade de Brest.png</v>
       </c>
     </row>
-    <row r="385" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A385" s="1" t="s">
         <v>7</v>
       </c>
@@ -20946,14 +20946,14 @@
         <v>1424</v>
       </c>
       <c r="N385" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O385" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Estuaire de Trieux.png</v>
       </c>
     </row>
-    <row r="386" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A386" s="1" t="s">
         <v>7</v>
       </c>
@@ -20982,14 +20982,14 @@
         <v>1427</v>
       </c>
       <c r="N386" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O386" s="23" t="str">
         <f t="shared" si="5"/>
         <v>DATA/logos/Baie de Veys.png</v>
       </c>
     </row>
-    <row r="387" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A387" s="1" t="s">
         <v>7</v>
       </c>
@@ -21018,14 +21018,14 @@
         <v>1430</v>
       </c>
       <c r="N387" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O387" s="23" t="str">
         <f t="shared" ref="O387:O388" si="6">"DATA/logos/" &amp; TEXT(E387,"jjj") &amp; ".png"</f>
         <v>DATA/logos/Anse du Cul du Loup.png</v>
       </c>
     </row>
-    <row r="388" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A388" s="1" t="s">
         <v>7</v>
       </c>
@@ -21054,7 +21054,7 @@
         <v>1433</v>
       </c>
       <c r="N388" s="32" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="O388" s="23" t="str">
         <f t="shared" si="6"/>

</xml_diff>

<commit_message>
duplication selection pour permettre carte dom tom
</commit_message>
<xml_diff>
--- a/Data/FairCarboN_Datas_Labo2.xlsx
+++ b/Data/FairCarboN_Datas_Labo2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719E8BB7-7507-4471-AA96-66CA07176114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F36882B6-52A3-4A7D-8999-0C7D40328AF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4117" uniqueCount="1435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4117" uniqueCount="1431">
   <si>
     <t>Acronyme PEPR</t>
   </si>
@@ -4366,9 +4366,6 @@
     <t>Austria</t>
   </si>
   <si>
-    <t>Nouvelle-Calédonie</t>
-  </si>
-  <si>
     <t>Germany</t>
   </si>
   <si>
@@ -4393,9 +4390,6 @@
     <t>Brazil</t>
   </si>
   <si>
-    <t>French Guiana</t>
-  </si>
-  <si>
     <t>Groenland</t>
   </si>
   <si>
@@ -4418,12 +4412,6 @@
   </si>
   <si>
     <t>Tunisia</t>
-  </si>
-  <si>
-    <t>Reunion Island</t>
-  </si>
-  <si>
-    <t>New Caledonia</t>
   </si>
   <si>
     <t>Etang de Sarrat</t>
@@ -4439,11 +4427,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -4620,10 +4615,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4631,61 +4626,61 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -4694,8 +4689,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4703,19 +4704,16 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4950,7 +4948,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:O469"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -5016,10 +5013,10 @@
         <v>1408</v>
       </c>
       <c r="O1" s="31" t="s">
-        <v>1419</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" ht="93.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1418</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="93.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -5067,7 +5064,7 @@
         <v>DATA/logos/AD2M.png</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="110" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" ht="110" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -5115,7 +5112,7 @@
         <v>DATA/logos/AGAP.png</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="114.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" ht="114.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -5163,7 +5160,7 @@
         <v>DATA/logos/AGAP.png</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="93" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" ht="93" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -5209,7 +5206,7 @@
         <v>DATA/logos/AGIR.png</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="93" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" ht="93" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -5255,7 +5252,7 @@
         <v>DATA/logos/AGIR.png</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="201.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" ht="201.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -5303,7 +5300,7 @@
         <v>DATA/logos/Agroécologie.png</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="101" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" ht="101" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -5351,7 +5348,7 @@
         <v>DATA/logos/Agroécologie.png</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="120.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" ht="120.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -5399,7 +5396,7 @@
         <v>DATA/logos/AIDA.png</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="118.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" ht="118.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>7</v>
       </c>
@@ -5447,7 +5444,7 @@
         <v>DATA/logos/AIDA.png</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="185" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" ht="185" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
@@ -5495,7 +5492,7 @@
         <v>DATA/logos/AMAP.png</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="409.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
@@ -5543,7 +5540,7 @@
         <v>DATA/logos/AMAP.png</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="31" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" ht="31" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
@@ -5585,7 +5582,7 @@
         <v>DATA/logos/ARVALIS.png</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="232" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" ht="232" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>7</v>
       </c>
@@ -5633,7 +5630,7 @@
         <v>DATA/logos/ASTRO.png</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>7</v>
       </c>
@@ -5679,7 +5676,7 @@
         <v>DATA/logos/BEF.png</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>7</v>
       </c>
@@ -5725,7 +5722,7 @@
         <v>DATA/logos/BEF.png</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>7</v>
       </c>
@@ -5771,7 +5768,7 @@
         <v>DATA/logos/BEF.png</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>7</v>
       </c>
@@ -5817,7 +5814,7 @@
         <v>DATA/logos/BEF.png</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>7</v>
       </c>
@@ -5863,7 +5860,7 @@
         <v>DATA/logos/BEF.png</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="108.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>7</v>
       </c>
@@ -5907,7 +5904,7 @@
         <v>DATA/logos/BETA.png</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="87.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" ht="87.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>7</v>
       </c>
@@ -5955,7 +5952,7 @@
         <v>DATA/logos/BIAM.png</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="92" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" ht="92" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>7</v>
       </c>
@@ -6003,7 +6000,7 @@
         <v>DATA/logos/BIAM.png</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="90" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>7</v>
       </c>
@@ -6051,7 +6048,7 @@
         <v>DATA/logos/BIAM.png</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="163.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" ht="163.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
@@ -6099,7 +6096,7 @@
         <v>DATA/logos/BioEcoAgro.png</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="135.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" ht="135.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>7</v>
       </c>
@@ -6147,7 +6144,7 @@
         <v>DATA/logos/BioEcoAgro.png</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="102.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" ht="102.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>7</v>
       </c>
@@ -6195,7 +6192,7 @@
         <v>DATA/logos/BIP.png</v>
       </c>
     </row>
-    <row r="27" spans="1:15" ht="27.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>7</v>
       </c>
@@ -6237,7 +6234,7 @@
         <v>DATA/logos/BMES.png</v>
       </c>
     </row>
-    <row r="28" spans="1:15" ht="59" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" ht="59" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>7</v>
       </c>
@@ -6283,7 +6280,7 @@
         <v>DATA/logos/BOREA.png</v>
       </c>
     </row>
-    <row r="29" spans="1:15" ht="77.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>7</v>
       </c>
@@ -6329,7 +6326,7 @@
         <v>DATA/logos/BOREA.png</v>
       </c>
     </row>
-    <row r="30" spans="1:15" ht="31" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" ht="31" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>7</v>
       </c>
@@ -6371,7 +6368,7 @@
         <v>DATA/logos/BOTANY.png</v>
       </c>
     </row>
-    <row r="31" spans="1:15" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>7</v>
       </c>
@@ -6411,7 +6408,7 @@
         <v>DATA/logos/CARBOFLUX.png</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>7</v>
       </c>
@@ -6457,7 +6454,7 @@
         <v>DATA/logos/CARRTEL.png</v>
       </c>
     </row>
-    <row r="33" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>7</v>
       </c>
@@ -6503,7 +6500,7 @@
         <v>DATA/logos/CARRTEL.png</v>
       </c>
     </row>
-    <row r="34" spans="1:15" ht="112.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:15" ht="112.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>7</v>
       </c>
@@ -6551,7 +6548,7 @@
         <v>DATA/logos/CEE-M.png</v>
       </c>
     </row>
-    <row r="35" spans="1:15" ht="171" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:15" ht="171" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>7</v>
       </c>
@@ -6599,7 +6596,7 @@
         <v>DATA/logos/CEFE.png</v>
       </c>
     </row>
-    <row r="36" spans="1:15" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:15" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>7</v>
       </c>
@@ -6645,7 +6642,7 @@
         <v>DATA/logos/CEFREM.png</v>
       </c>
     </row>
-    <row r="37" spans="1:15" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:15" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>7</v>
       </c>
@@ -6691,7 +6688,7 @@
         <v>DATA/logos/CEREGE.png</v>
       </c>
     </row>
-    <row r="38" spans="1:15" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:15" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>7</v>
       </c>
@@ -6737,7 +6734,7 @@
         <v>DATA/logos/CESBIO.png</v>
       </c>
     </row>
-    <row r="39" spans="1:15" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:15" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>7</v>
       </c>
@@ -6783,7 +6780,7 @@
         <v>DATA/logos/CESBIO.png</v>
       </c>
     </row>
-    <row r="40" spans="1:15" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>7</v>
       </c>
@@ -6829,7 +6826,7 @@
         <v>DATA/logos/CMH.png</v>
       </c>
     </row>
-    <row r="41" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>7</v>
       </c>
@@ -6875,7 +6872,7 @@
         <v>DATA/logos/CNRM.png</v>
       </c>
     </row>
-    <row r="42" spans="1:15" ht="63.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:15" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>7</v>
       </c>
@@ -6921,7 +6918,7 @@
         <v>DATA/logos/CNRM.png</v>
       </c>
     </row>
-    <row r="43" spans="1:15" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:15" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>7</v>
       </c>
@@ -6967,7 +6964,7 @@
         <v>DATA/logos/CRBE.png</v>
       </c>
     </row>
-    <row r="44" spans="1:15" ht="95.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:15" ht="95.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>7</v>
       </c>
@@ -7013,7 +7010,7 @@
         <v>DATA/logos/CRBE.png</v>
       </c>
     </row>
-    <row r="45" spans="1:15" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:15" ht="87" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>7</v>
       </c>
@@ -7061,7 +7058,7 @@
         <v>DATA/logos/CRJ.png</v>
       </c>
     </row>
-    <row r="46" spans="1:15" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:15" ht="85" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>7</v>
       </c>
@@ -7109,7 +7106,7 @@
         <v>DATA/logos/DIADE.png</v>
       </c>
     </row>
-    <row r="47" spans="1:15" ht="156.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:15" ht="156.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>7</v>
       </c>
@@ -7157,7 +7154,7 @@
         <v>DATA/logos/Eco&amp;Sols.png</v>
       </c>
     </row>
-    <row r="48" spans="1:15" ht="183.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:15" ht="183.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>7</v>
       </c>
@@ -7205,7 +7202,7 @@
         <v>DATA/logos/Eco&amp;Sols.png</v>
       </c>
     </row>
-    <row r="49" spans="1:15" ht="137" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:15" ht="137" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>7</v>
       </c>
@@ -7253,7 +7250,7 @@
         <v>DATA/logos/Eco&amp;Sols.png</v>
       </c>
     </row>
-    <row r="50" spans="1:15" ht="146" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:15" ht="146" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>7</v>
       </c>
@@ -7301,7 +7298,7 @@
         <v>DATA/logos/Eco&amp;Sols.png</v>
       </c>
     </row>
-    <row r="51" spans="1:15" ht="109.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:15" ht="109.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>7</v>
       </c>
@@ -7349,7 +7346,7 @@
         <v>DATA/logos/Eco&amp;Sols.png</v>
       </c>
     </row>
-    <row r="52" spans="1:15" ht="114.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:15" ht="114.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>7</v>
       </c>
@@ -7397,7 +7394,7 @@
         <v>DATA/logos/Eco&amp;Sols.png</v>
       </c>
     </row>
-    <row r="53" spans="1:15" ht="114.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:15" ht="114.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>7</v>
       </c>
@@ -7445,7 +7442,7 @@
         <v>DATA/logos/Eco&amp;Sols.png</v>
       </c>
     </row>
-    <row r="54" spans="1:15" ht="131.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:15" ht="131.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>7</v>
       </c>
@@ -7493,7 +7490,7 @@
         <v>DATA/logos/ECOBIO.png</v>
       </c>
     </row>
-    <row r="55" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>7</v>
       </c>
@@ -7539,7 +7536,7 @@
         <v>DATA/logos/ECODIV.png</v>
       </c>
     </row>
-    <row r="56" spans="1:15" ht="111" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:15" ht="111" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>7</v>
       </c>
@@ -7587,7 +7584,7 @@
         <v>DATA/logos/ECOSYS.png</v>
       </c>
     </row>
-    <row r="57" spans="1:15" ht="115" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:15" ht="115" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>7</v>
       </c>
@@ -7635,7 +7632,7 @@
         <v>DATA/logos/ECOSYS.png</v>
       </c>
     </row>
-    <row r="58" spans="1:15" ht="157.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:15" ht="157.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>7</v>
       </c>
@@ -7683,7 +7680,7 @@
         <v>DATA/logos/ECOSYS.png</v>
       </c>
     </row>
-    <row r="59" spans="1:15" ht="127.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:15" ht="127.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>7</v>
       </c>
@@ -7731,7 +7728,7 @@
         <v>DATA/logos/ECOSYS.png</v>
       </c>
     </row>
-    <row r="60" spans="1:15" ht="163.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:15" ht="163.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>7</v>
       </c>
@@ -7779,7 +7776,7 @@
         <v>DATA/logos/ECOSYS.png</v>
       </c>
     </row>
-    <row r="61" spans="1:15" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>7</v>
       </c>
@@ -7821,7 +7818,7 @@
         <v>DATA/logos/EDF.png</v>
       </c>
     </row>
-    <row r="62" spans="1:15" ht="145" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:15" ht="145" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>7</v>
       </c>
@@ -7869,7 +7866,7 @@
         <v>DATA/logos/EDYTEM.png</v>
       </c>
     </row>
-    <row r="63" spans="1:15" ht="145" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:15" ht="145" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>7</v>
       </c>
@@ -7917,7 +7914,7 @@
         <v>DATA/logos/EDYTEM.png</v>
       </c>
     </row>
-    <row r="64" spans="1:15" ht="221" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:15" ht="221" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>7</v>
       </c>
@@ -7965,7 +7962,7 @@
         <v>DATA/logos/EMMAH.png</v>
       </c>
     </row>
-    <row r="65" spans="1:15" ht="225" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:15" ht="225" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>7</v>
       </c>
@@ -8013,7 +8010,7 @@
         <v>DATA/logos/EMMAH.png</v>
       </c>
     </row>
-    <row r="66" spans="1:15" ht="77.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:15" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>7</v>
       </c>
@@ -8059,7 +8056,7 @@
         <v>DATA/logos/EPOC.png</v>
       </c>
     </row>
-    <row r="67" spans="1:15" ht="77.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:15" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>7</v>
       </c>
@@ -8105,7 +8102,7 @@
         <v>DATA/logos/EPOC.png</v>
       </c>
     </row>
-    <row r="68" spans="1:15" ht="77.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:15" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>7</v>
       </c>
@@ -8151,7 +8148,7 @@
         <v>DATA/logos/EPOC.png</v>
       </c>
     </row>
-    <row r="69" spans="1:15" ht="106.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:15" ht="106.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>7</v>
       </c>
@@ -8199,7 +8196,7 @@
         <v>DATA/logos/ESE.png</v>
       </c>
     </row>
-    <row r="70" spans="1:15" ht="147.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:15" ht="147.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>7</v>
       </c>
@@ -8247,7 +8244,7 @@
         <v>DATA/logos/ESE.png</v>
       </c>
     </row>
-    <row r="71" spans="1:15" ht="150.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:15" ht="150.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>7</v>
       </c>
@@ -8295,7 +8292,7 @@
         <v>DATA/logos/FARE.png</v>
       </c>
     </row>
-    <row r="72" spans="1:15" ht="105.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:15" ht="105.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>7</v>
       </c>
@@ -8343,7 +8340,7 @@
         <v>DATA/logos/FARE.png</v>
       </c>
     </row>
-    <row r="73" spans="1:15" ht="141.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:15" ht="141.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>7</v>
       </c>
@@ -8391,7 +8388,7 @@
         <v>DATA/logos/FARE.png</v>
       </c>
     </row>
-    <row r="74" spans="1:15" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:15" ht="87" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>7</v>
       </c>
@@ -8439,7 +8436,7 @@
         <v>DATA/logos/GAEL.png</v>
       </c>
     </row>
-    <row r="75" spans="1:15" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:15" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>7</v>
       </c>
@@ -8485,7 +8482,7 @@
         <v>DATA/logos/GEODE.png</v>
       </c>
     </row>
-    <row r="76" spans="1:15" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:15" ht="87" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>7</v>
       </c>
@@ -8531,7 +8528,7 @@
         <v>DATA/logos/GEOPS.png</v>
       </c>
     </row>
-    <row r="77" spans="1:15" ht="46.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:15" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>7</v>
       </c>
@@ -8545,7 +8542,7 @@
         <v>659</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>1434</v>
+        <v>1430</v>
       </c>
       <c r="F77" s="13"/>
       <c r="G77" s="13" t="s">
@@ -8575,7 +8572,7 @@
         <v>DATA/logos/GS Fontainebleau.png</v>
       </c>
     </row>
-    <row r="78" spans="1:15" ht="131" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:15" ht="131" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>7</v>
       </c>
@@ -8589,7 +8586,7 @@
         <v>196</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>1433</v>
+        <v>1429</v>
       </c>
       <c r="F78" s="5" t="s">
         <v>663</v>
@@ -8623,7 +8620,7 @@
         <v>DATA/logos/GS Rennes.png</v>
       </c>
     </row>
-    <row r="79" spans="1:15" ht="133.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:15" ht="133.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>7</v>
       </c>
@@ -8637,7 +8634,7 @@
         <v>196</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>1433</v>
+        <v>1429</v>
       </c>
       <c r="F79" s="5" t="s">
         <v>663</v>
@@ -8671,7 +8668,7 @@
         <v>DATA/logos/GS Rennes.png</v>
       </c>
     </row>
-    <row r="80" spans="1:15" ht="62" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:15" ht="62" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>7</v>
       </c>
@@ -8717,7 +8714,7 @@
         <v>DATA/logos/GET.png</v>
       </c>
     </row>
-    <row r="81" spans="1:15" ht="62" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:15" ht="62" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>7</v>
       </c>
@@ -8763,7 +8760,7 @@
         <v>DATA/logos/GET.png</v>
       </c>
     </row>
-    <row r="82" spans="1:15" ht="62" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:15" ht="62" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>7</v>
       </c>
@@ -8809,7 +8806,7 @@
         <v>DATA/logos/GET.png</v>
       </c>
     </row>
-    <row r="83" spans="1:15" ht="132.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:15" ht="132.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>7</v>
       </c>
@@ -8857,7 +8854,7 @@
         <v>DATA/logos/HSM.png</v>
       </c>
     </row>
-    <row r="84" spans="1:15" ht="150.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:15" ht="150.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>7</v>
       </c>
@@ -8905,7 +8902,7 @@
         <v>DATA/logos/IAM.png</v>
       </c>
     </row>
-    <row r="85" spans="1:15" ht="126.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:15" ht="126.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>7</v>
       </c>
@@ -8953,7 +8950,7 @@
         <v>DATA/logos/IATE.png</v>
       </c>
     </row>
-    <row r="86" spans="1:15" ht="159" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:15" ht="159" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>7</v>
       </c>
@@ -9001,7 +8998,7 @@
         <v>DATA/logos/iEES.png</v>
       </c>
     </row>
-    <row r="87" spans="1:15" ht="132.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:15" ht="132.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>7</v>
       </c>
@@ -9049,7 +9046,7 @@
         <v>DATA/logos/iEES.png</v>
       </c>
     </row>
-    <row r="88" spans="1:15" ht="94.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:15" ht="94.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>7</v>
       </c>
@@ -9097,7 +9094,7 @@
         <v>DATA/logos/iEES.png</v>
       </c>
     </row>
-    <row r="89" spans="1:15" ht="161" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:15" ht="161" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>7</v>
       </c>
@@ -9145,7 +9142,7 @@
         <v>DATA/logos/iEES.png</v>
       </c>
     </row>
-    <row r="90" spans="1:15" ht="132" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:15" ht="132" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>7</v>
       </c>
@@ -9193,7 +9190,7 @@
         <v>DATA/logos/iEES.png</v>
       </c>
     </row>
-    <row r="91" spans="1:15" ht="134" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:15" ht="134" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>7</v>
       </c>
@@ -9241,7 +9238,7 @@
         <v>DATA/logos/iEES.png</v>
       </c>
     </row>
-    <row r="92" spans="1:15" ht="125" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:15" ht="125" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>7</v>
       </c>
@@ -9289,7 +9286,7 @@
         <v>DATA/logos/iEES.png</v>
       </c>
     </row>
-    <row r="93" spans="1:15" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:15" ht="102" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>7</v>
       </c>
@@ -9337,7 +9334,7 @@
         <v>DATA/logos/IGE.png</v>
       </c>
     </row>
-    <row r="94" spans="1:15" ht="112.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:15" ht="112.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>7</v>
       </c>
@@ -9385,7 +9382,7 @@
         <v>DATA/logos/IGE.png</v>
       </c>
     </row>
-    <row r="95" spans="1:15" ht="147.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:15" ht="147.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>7</v>
       </c>
@@ -9433,7 +9430,7 @@
         <v>DATA/logos/IGE.png</v>
       </c>
     </row>
-    <row r="96" spans="1:15" ht="129.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:15" ht="129.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>7</v>
       </c>
@@ -9481,7 +9478,7 @@
         <v>DATA/logos/IGE.png</v>
       </c>
     </row>
-    <row r="97" spans="1:15" ht="142" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:15" ht="142" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>7</v>
       </c>
@@ -9529,7 +9526,7 @@
         <v>DATA/logos/IJPB.png</v>
       </c>
     </row>
-    <row r="98" spans="1:15" ht="104" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:15" ht="104" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>7</v>
       </c>
@@ -9577,7 +9574,7 @@
         <v>DATA/logos/IMBE.png</v>
       </c>
     </row>
-    <row r="99" spans="1:15" ht="46.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:15" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>7</v>
       </c>
@@ -9623,7 +9620,7 @@
         <v>DATA/logos/IMM.png</v>
       </c>
     </row>
-    <row r="100" spans="1:15" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:15" ht="87" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>7</v>
       </c>
@@ -9669,7 +9666,7 @@
         <v>DATA/logos/Info&amp;Sols.png</v>
       </c>
     </row>
-    <row r="101" spans="1:15" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>7</v>
       </c>
@@ -9711,7 +9708,7 @@
         <v>DATA/logos/INRAE.png</v>
       </c>
     </row>
-    <row r="102" spans="1:15" ht="165.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:15" ht="165.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>7</v>
       </c>
@@ -9759,7 +9756,7 @@
         <v>DATA/logos/IPGP.png</v>
       </c>
     </row>
-    <row r="103" spans="1:15" ht="79.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:15" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>7</v>
       </c>
@@ -9807,7 +9804,7 @@
         <v>DATA/logos/IPGP.png</v>
       </c>
     </row>
-    <row r="104" spans="1:15" ht="48" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:15" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>7</v>
       </c>
@@ -9855,7 +9852,7 @@
         <v>DATA/logos/IRIT.png</v>
       </c>
     </row>
-    <row r="105" spans="1:15" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:15" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>7</v>
       </c>
@@ -9896,14 +9893,14 @@
         <v>389</v>
       </c>
       <c r="N105" s="1" t="s">
-        <v>1412</v>
+        <v>1409</v>
       </c>
       <c r="O105" s="23" t="str">
         <f t="shared" si="1"/>
         <v>DATA/logos/ISEA.png</v>
       </c>
     </row>
-    <row r="106" spans="1:15" ht="177.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:15" ht="177.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>7</v>
       </c>
@@ -9951,7 +9948,7 @@
         <v>DATA/logos/ISEM.png</v>
       </c>
     </row>
-    <row r="107" spans="1:15" ht="197" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:15" ht="197" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>7</v>
       </c>
@@ -9999,7 +9996,7 @@
         <v>DATA/logos/ISOMer.png</v>
       </c>
     </row>
-    <row r="108" spans="1:15" ht="204" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:15" ht="204" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>7</v>
       </c>
@@ -10047,7 +10044,7 @@
         <v>DATA/logos/ISOMer.png</v>
       </c>
     </row>
-    <row r="109" spans="1:15" ht="182.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:15" ht="182.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>7</v>
       </c>
@@ -10095,7 +10092,7 @@
         <v>DATA/logos/ISPA.png</v>
       </c>
     </row>
-    <row r="110" spans="1:15" ht="126" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:15" ht="126" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>7</v>
       </c>
@@ -10143,7 +10140,7 @@
         <v>DATA/logos/ISPA.png</v>
       </c>
     </row>
-    <row r="111" spans="1:15" ht="163" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:15" ht="163" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>7</v>
       </c>
@@ -10191,7 +10188,7 @@
         <v>DATA/logos/ISPA.png</v>
       </c>
     </row>
-    <row r="112" spans="1:15" ht="131" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:15" ht="131" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>7</v>
       </c>
@@ -10239,7 +10236,7 @@
         <v>DATA/logos/iSTeP.png</v>
       </c>
     </row>
-    <row r="113" spans="1:15" ht="121.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:15" ht="121.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>7</v>
       </c>
@@ -10287,7 +10284,7 @@
         <v>DATA/logos/iSTeP.png</v>
       </c>
     </row>
-    <row r="114" spans="1:15" ht="117.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:15" ht="117.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>7</v>
       </c>
@@ -10335,7 +10332,7 @@
         <v>DATA/logos/iSTeP.png</v>
       </c>
     </row>
-    <row r="115" spans="1:15" ht="143" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:15" ht="143" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>7</v>
       </c>
@@ -10383,7 +10380,7 @@
         <v>DATA/logos/ISTERRE.png</v>
       </c>
     </row>
-    <row r="116" spans="1:15" ht="186.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:15" ht="186.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>7</v>
       </c>
@@ -10431,7 +10428,7 @@
         <v>DATA/logos/ISTO.png</v>
       </c>
     </row>
-    <row r="117" spans="1:15" ht="157.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:15" ht="157.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>7</v>
       </c>
@@ -10479,7 +10476,7 @@
         <v>DATA/logos/ISTO.png</v>
       </c>
     </row>
-    <row r="118" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>7</v>
       </c>
@@ -10525,7 +10522,7 @@
         <v>DATA/logos/ITAP.png</v>
       </c>
     </row>
-    <row r="119" spans="1:15" ht="93" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:15" ht="93" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>7</v>
       </c>
@@ -10573,7 +10570,7 @@
         <v>DATA/logos/LAE.png</v>
       </c>
     </row>
-    <row r="120" spans="1:15" ht="232" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:15" ht="232" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>7</v>
       </c>
@@ -10621,7 +10618,7 @@
         <v>DATA/logos/LAE.png</v>
       </c>
     </row>
-    <row r="121" spans="1:15" ht="51.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:15" ht="51.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>7</v>
       </c>
@@ -10667,7 +10664,7 @@
         <v>DATA/logos/LBE.png</v>
       </c>
     </row>
-    <row r="122" spans="1:15" ht="179" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:15" ht="179" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>7</v>
       </c>
@@ -10715,7 +10712,7 @@
         <v>DATA/logos/LCB.png</v>
       </c>
     </row>
-    <row r="123" spans="1:15" ht="161" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:15" ht="161" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>7</v>
       </c>
@@ -10763,7 +10760,7 @@
         <v>DATA/logos/LCE.png</v>
       </c>
     </row>
-    <row r="124" spans="1:15" ht="181.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:15" ht="181.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>7</v>
       </c>
@@ -10811,7 +10808,7 @@
         <v>DATA/logos/LCE.png</v>
       </c>
     </row>
-    <row r="125" spans="1:15" ht="132" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:15" ht="132" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>7</v>
       </c>
@@ -10859,7 +10856,7 @@
         <v>DATA/logos/LEHNA.png</v>
       </c>
     </row>
-    <row r="126" spans="1:15" ht="157.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:15" ht="157.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>7</v>
       </c>
@@ -10907,7 +10904,7 @@
         <v>DATA/logos/LEHNA.png</v>
       </c>
     </row>
-    <row r="127" spans="1:15" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:15" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>7</v>
       </c>
@@ -10955,7 +10952,7 @@
         <v>DATA/logos/LEM.png</v>
       </c>
     </row>
-    <row r="128" spans="1:15" ht="195" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:15" ht="195" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>7</v>
       </c>
@@ -11003,7 +11000,7 @@
         <v>DATA/logos/LEMAR.png</v>
       </c>
     </row>
-    <row r="129" spans="1:15" ht="213" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:15" ht="213" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>7</v>
       </c>
@@ -11051,7 +11048,7 @@
         <v>DATA/logos/LEMAR.png</v>
       </c>
     </row>
-    <row r="130" spans="1:15" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>7</v>
       </c>
@@ -11095,7 +11092,7 @@
         <v>DATA/logos/LERPC.png</v>
       </c>
     </row>
-    <row r="131" spans="1:15" ht="145" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:15" ht="145" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>7</v>
       </c>
@@ -11143,7 +11140,7 @@
         <v>DATA/logos/LESSEM.png</v>
       </c>
     </row>
-    <row r="132" spans="1:15" ht="48.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:15" ht="48.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>7</v>
       </c>
@@ -11191,7 +11188,7 @@
         <v>DATA/logos/LETG.png</v>
       </c>
     </row>
-    <row r="133" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>7</v>
       </c>
@@ -11237,7 +11234,7 @@
         <v>DATA/logos/LG-ENS.png</v>
       </c>
     </row>
-    <row r="134" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>7</v>
       </c>
@@ -11283,7 +11280,7 @@
         <v>DATA/logos/LG-ENS.png</v>
       </c>
     </row>
-    <row r="135" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>7</v>
       </c>
@@ -11329,7 +11326,7 @@
         <v>DATA/logos/LG-ENS.png</v>
       </c>
     </row>
-    <row r="136" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>7</v>
       </c>
@@ -11375,7 +11372,7 @@
         <v>DATA/logos/LG-ENS.png</v>
       </c>
     </row>
-    <row r="137" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>7</v>
       </c>
@@ -11421,7 +11418,7 @@
         <v>DATA/logos/LG-ENS.png</v>
       </c>
     </row>
-    <row r="138" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>7</v>
       </c>
@@ -11467,7 +11464,7 @@
         <v>DATA/logos/LG-ENS.png</v>
       </c>
     </row>
-    <row r="139" spans="1:15" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>7</v>
       </c>
@@ -11513,7 +11510,7 @@
         <v>DATA/logos/LG-ENS.png</v>
       </c>
     </row>
-    <row r="140" spans="1:15" ht="101.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:15" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>7</v>
       </c>
@@ -11561,7 +11558,7 @@
         <v>DATA/logos/LIED.png</v>
       </c>
     </row>
-    <row r="141" spans="1:15" ht="107" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:15" ht="107" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>7</v>
       </c>
@@ -11607,7 +11604,7 @@
         <v>DATA/logos/LIENSs.png</v>
       </c>
     </row>
-    <row r="142" spans="1:15" ht="155" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:15" ht="155" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>7</v>
       </c>
@@ -11653,7 +11650,7 @@
         <v>DATA/logos/LIENSs.png</v>
       </c>
     </row>
-    <row r="143" spans="1:15" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:15" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>7</v>
       </c>
@@ -11695,7 +11692,7 @@
         <v>DATA/logos/LIF.png</v>
       </c>
     </row>
-    <row r="144" spans="1:15" ht="198.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:15" ht="198.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>7</v>
       </c>
@@ -11743,7 +11740,7 @@
         <v>DATA/logos/LIRMM.png</v>
       </c>
     </row>
-    <row r="145" spans="1:15" ht="46.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:15" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>7</v>
       </c>
@@ -11789,7 +11786,7 @@
         <v>DATA/logos/LISAH.png</v>
       </c>
     </row>
-    <row r="146" spans="1:15" ht="46.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:15" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>7</v>
       </c>
@@ -11835,7 +11832,7 @@
         <v>DATA/logos/LISAH.png</v>
       </c>
     </row>
-    <row r="147" spans="1:15" ht="46.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:15" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>7</v>
       </c>
@@ -11881,7 +11878,7 @@
         <v>DATA/logos/LISAH.png</v>
       </c>
     </row>
-    <row r="148" spans="1:15" ht="46.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:15" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>7</v>
       </c>
@@ -11927,7 +11924,7 @@
         <v>DATA/logos/LISAH.png</v>
       </c>
     </row>
-    <row r="149" spans="1:15" ht="46.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:15" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>7</v>
       </c>
@@ -11973,7 +11970,7 @@
         <v>DATA/logos/LISAH.png</v>
       </c>
     </row>
-    <row r="150" spans="1:15" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:15" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>7</v>
       </c>
@@ -12019,7 +12016,7 @@
         <v>DATA/logos/LISC.png</v>
       </c>
     </row>
-    <row r="151" spans="1:15" ht="93" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:15" ht="93" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>7</v>
       </c>
@@ -12063,7 +12060,7 @@
         <v>DATA/logos/LMD.png</v>
       </c>
     </row>
-    <row r="152" spans="1:15" ht="112.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:15" ht="112.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>7</v>
       </c>
@@ -12111,7 +12108,7 @@
         <v>DATA/logos/LOG.png</v>
       </c>
     </row>
-    <row r="153" spans="1:15" ht="220.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:15" ht="220.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>7</v>
       </c>
@@ -12159,7 +12156,7 @@
         <v>DATA/logos/LOG.png</v>
       </c>
     </row>
-    <row r="154" spans="1:15" ht="248" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:15" ht="248" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>7</v>
       </c>
@@ -12207,7 +12204,7 @@
         <v>DATA/logos/LPC2E.png</v>
       </c>
     </row>
-    <row r="155" spans="1:15" ht="108.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:15" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>7</v>
       </c>
@@ -12253,7 +12250,7 @@
         <v>DATA/logos/LPG.png</v>
       </c>
     </row>
-    <row r="156" spans="1:15" ht="108.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:15" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>7</v>
       </c>
@@ -12299,7 +12296,7 @@
         <v>DATA/logos/LPG.png</v>
       </c>
     </row>
-    <row r="157" spans="1:15" ht="108.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:15" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>7</v>
       </c>
@@ -12345,7 +12342,7 @@
         <v>DATA/logos/LPG.png</v>
       </c>
     </row>
-    <row r="158" spans="1:15" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:15" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>7</v>
       </c>
@@ -12391,7 +12388,7 @@
         <v>DATA/logos/LSCE.png</v>
       </c>
     </row>
-    <row r="159" spans="1:15" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:15" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>7</v>
       </c>
@@ -12437,7 +12434,7 @@
         <v>DATA/logos/LSCE.png</v>
       </c>
     </row>
-    <row r="160" spans="1:15" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:15" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>7</v>
       </c>
@@ -12483,7 +12480,7 @@
         <v>DATA/logos/LSCE.png</v>
       </c>
     </row>
-    <row r="161" spans="1:15" ht="130.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:15" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>7</v>
       </c>
@@ -12529,7 +12526,7 @@
         <v>DATA/logos/LSCE.png</v>
       </c>
     </row>
-    <row r="162" spans="1:15" ht="171" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:15" ht="171" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>7</v>
       </c>
@@ -12577,7 +12574,7 @@
         <v>DATA/logos/LUSAC.png</v>
       </c>
     </row>
-    <row r="163" spans="1:15" ht="172.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:15" ht="172.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
         <v>7</v>
       </c>
@@ -12625,7 +12622,7 @@
         <v>DATA/logos/M2C.png</v>
       </c>
     </row>
-    <row r="164" spans="1:15" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>7</v>
       </c>
@@ -12660,14 +12657,14 @@
         <v>834</v>
       </c>
       <c r="N164" s="1" t="s">
-        <v>1413</v>
+        <v>1412</v>
       </c>
       <c r="O164" s="23" t="str">
         <f t="shared" si="2"/>
         <v>DATA/logos/MAXPLANCK.png</v>
       </c>
     </row>
-    <row r="165" spans="1:15" ht="135" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:15" ht="135" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>7</v>
       </c>
@@ -12715,7 +12712,7 @@
         <v>DATA/logos/METIS.png</v>
       </c>
     </row>
-    <row r="166" spans="1:15" ht="100.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:15" ht="100.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>7</v>
       </c>
@@ -12763,7 +12760,7 @@
         <v>DATA/logos/METIS.png</v>
       </c>
     </row>
-    <row r="167" spans="1:15" ht="115.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:15" ht="115.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>7</v>
       </c>
@@ -12811,7 +12808,7 @@
         <v>DATA/logos/METIS.png</v>
       </c>
     </row>
-    <row r="168" spans="1:15" ht="124.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:15" ht="124.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>7</v>
       </c>
@@ -12859,7 +12856,7 @@
         <v>DATA/logos/METIS.png</v>
       </c>
     </row>
-    <row r="169" spans="1:15" ht="166.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:15" ht="166.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
         <v>7</v>
       </c>
@@ -12907,7 +12904,7 @@
         <v>DATA/logos/OPAALE.png</v>
       </c>
     </row>
-    <row r="170" spans="1:15" ht="77.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:15" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>7</v>
       </c>
@@ -12953,7 +12950,7 @@
         <v>DATA/logos/PjSE.png</v>
       </c>
     </row>
-    <row r="171" spans="1:15" ht="77.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:15" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>7</v>
       </c>
@@ -12999,7 +12996,7 @@
         <v>DATA/logos/PjSE.png</v>
       </c>
     </row>
-    <row r="172" spans="1:15" ht="122.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:15" ht="122.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>7</v>
       </c>
@@ -13047,7 +13044,7 @@
         <v>DATA/logos/PSAE.png</v>
       </c>
     </row>
-    <row r="173" spans="1:15" ht="319" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:15" ht="319" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>7</v>
       </c>
@@ -13095,7 +13092,7 @@
         <v>DATA/logos/PSAE.png</v>
       </c>
     </row>
-    <row r="174" spans="1:15" ht="62" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:15" ht="62" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>7</v>
       </c>
@@ -13139,7 +13136,7 @@
         <v>DATA/logos/PSE.png</v>
       </c>
     </row>
-    <row r="175" spans="1:15" ht="232" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:15" ht="232" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>7</v>
       </c>
@@ -13187,7 +13184,7 @@
         <v>DATA/logos/RECOVER.png</v>
       </c>
     </row>
-    <row r="176" spans="1:15" ht="155" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:15" ht="155" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>7</v>
       </c>
@@ -13233,7 +13230,7 @@
         <v>DATA/logos/Recyclage&amp;Risques.png</v>
       </c>
     </row>
-    <row r="177" spans="1:15" ht="155" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:15" ht="155" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>7</v>
       </c>
@@ -13279,7 +13276,7 @@
         <v>DATA/logos/Recyclage&amp;Risques.png</v>
       </c>
     </row>
-    <row r="178" spans="1:15" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:15" ht="87" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>7</v>
       </c>
@@ -13323,7 +13320,7 @@
         <v>DATA/logos/RiverLy.png</v>
       </c>
     </row>
-    <row r="179" spans="1:15" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>7</v>
       </c>
@@ -13369,7 +13366,7 @@
         <v>DATA/logos/SAS.png</v>
       </c>
     </row>
-    <row r="180" spans="1:15" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>7</v>
       </c>
@@ -13415,7 +13412,7 @@
         <v>DATA/logos/SAS.png</v>
       </c>
     </row>
-    <row r="181" spans="1:15" ht="103.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:15" ht="103.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>7</v>
       </c>
@@ -13463,7 +13460,7 @@
         <v>DATA/logos/SELMET.png</v>
       </c>
     </row>
-    <row r="182" spans="1:15" ht="118.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:15" ht="118.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>7</v>
       </c>
@@ -13511,7 +13508,7 @@
         <v>DATA/logos/SELMET.png</v>
       </c>
     </row>
-    <row r="183" spans="1:15" ht="147" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:15" ht="147" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>7</v>
       </c>
@@ -13559,7 +13556,7 @@
         <v>DATA/logos/SELMET.png</v>
       </c>
     </row>
-    <row r="184" spans="1:15" s="2" customFormat="1" ht="120" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:15" s="2" customFormat="1" ht="120" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>7</v>
       </c>
@@ -13607,7 +13604,7 @@
         <v>DATA/logos/SILVA.png</v>
       </c>
     </row>
-    <row r="185" spans="1:15" s="2" customFormat="1" ht="148.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:15" s="2" customFormat="1" ht="148.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>7</v>
       </c>
@@ -13655,7 +13652,7 @@
         <v>DATA/logos/SILVA.png</v>
       </c>
     </row>
-    <row r="186" spans="1:15" s="2" customFormat="1" ht="246.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:15" s="2" customFormat="1" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>7</v>
       </c>
@@ -13703,7 +13700,7 @@
         <v>DATA/logos/SILVA.png</v>
       </c>
     </row>
-    <row r="187" spans="1:15" s="2" customFormat="1" ht="62" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:15" s="2" customFormat="1" ht="62" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>7</v>
       </c>
@@ -13749,7 +13746,7 @@
         <v>DATA/logos/SMART-LERECO.png</v>
       </c>
     </row>
-    <row r="188" spans="1:15" s="2" customFormat="1" ht="62" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:15" s="2" customFormat="1" ht="62" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>7</v>
       </c>
@@ -13795,7 +13792,7 @@
         <v>DATA/logos/SMART-LERECO.png</v>
       </c>
     </row>
-    <row r="189" spans="1:15" s="2" customFormat="1" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:15" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>7</v>
       </c>
@@ -13839,7 +13836,7 @@
         <v>DATA/logos/STLO.png</v>
       </c>
     </row>
-    <row r="190" spans="1:15" s="2" customFormat="1" ht="211.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:15" s="2" customFormat="1" ht="211.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>7</v>
       </c>
@@ -13887,7 +13884,7 @@
         <v>DATA/logos/TBI.png</v>
       </c>
     </row>
-    <row r="191" spans="1:15" s="2" customFormat="1" ht="108.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:15" s="2" customFormat="1" ht="108.5" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>7</v>
       </c>
@@ -13935,7 +13932,7 @@
         <v>DATA/logos/TSE - R.png</v>
       </c>
     </row>
-    <row r="192" spans="1:15" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>7</v>
       </c>
@@ -13970,14 +13967,14 @@
         <v>898</v>
       </c>
       <c r="N192" s="1" t="s">
-        <v>1414</v>
+        <v>1413</v>
       </c>
       <c r="O192" s="23" t="str">
         <f t="shared" si="2"/>
         <v>DATA/logos/UNESCO.png</v>
       </c>
     </row>
-    <row r="193" spans="1:15" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:15" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A193" s="1" t="s">
         <v>7</v>
       </c>
@@ -14023,7 +14020,7 @@
         <v>DATA/logos/UREP.png</v>
       </c>
     </row>
-    <row r="194" spans="1:15" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:15" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>7</v>
       </c>
@@ -14069,7 +14066,7 @@
         <v>DATA/logos/URFM.png</v>
       </c>
     </row>
-    <row r="195" spans="1:15" s="2" customFormat="1" ht="58" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:15" s="2" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>7</v>
       </c>
@@ -14115,7 +14112,7 @@
         <v>DATA/logos/URFM.png</v>
       </c>
     </row>
-    <row r="196" spans="1:15" s="2" customFormat="1" ht="72.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:15" s="2" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>7</v>
       </c>
@@ -14148,14 +14145,14 @@
         <v>908</v>
       </c>
       <c r="N196" s="1" t="s">
-        <v>1415</v>
+        <v>1414</v>
       </c>
       <c r="O196" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/CARDEC.png</v>
       </c>
     </row>
-    <row r="197" spans="1:15" s="2" customFormat="1" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:15" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>7</v>
       </c>
@@ -14197,7 +14194,7 @@
         <v>DATA/logos/ELI.png</v>
       </c>
     </row>
-    <row r="198" spans="1:15" s="2" customFormat="1" ht="46.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:15" s="2" customFormat="1" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>7</v>
       </c>
@@ -14236,14 +14233,14 @@
         <v>915</v>
       </c>
       <c r="N198" s="1" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
       <c r="O198" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/LMI-IESOL.png</v>
       </c>
     </row>
-    <row r="199" spans="1:15" s="2" customFormat="1" ht="46.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:15" s="2" customFormat="1" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>7</v>
       </c>
@@ -14276,14 +14273,14 @@
         <v>920</v>
       </c>
       <c r="N199" s="1" t="s">
-        <v>1417</v>
+        <v>1416</v>
       </c>
       <c r="O199" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/SFRI.png</v>
       </c>
     </row>
-    <row r="200" spans="1:15" s="2" customFormat="1" ht="159.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:15" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>7</v>
       </c>
@@ -14324,14 +14321,14 @@
         <v>915</v>
       </c>
       <c r="N200" s="1" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
       <c r="O200" s="23" t="str">
         <f t="shared" si="3"/>
         <v>DATA/logos/UMMISCO_UCAD.png</v>
       </c>
     </row>
-    <row r="201" spans="1:15" s="2" customFormat="1" ht="87" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:15" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>7</v>
       </c>
@@ -14362,7 +14359,7 @@
         <v>928</v>
       </c>
       <c r="N201" s="1" t="s">
-        <v>1418</v>
+        <v>1417</v>
       </c>
       <c r="O201" s="23" t="str">
         <f t="shared" si="3"/>
@@ -15262,7 +15259,7 @@
         <v>1004</v>
       </c>
       <c r="N226" s="1" t="s">
-        <v>1420</v>
+        <v>1419</v>
       </c>
       <c r="O226" s="23" t="str">
         <f t="shared" si="3"/>
@@ -15442,7 +15439,7 @@
         <v>1019</v>
       </c>
       <c r="N231" s="1" t="s">
-        <v>1417</v>
+        <v>1416</v>
       </c>
       <c r="O231" s="23" t="str">
         <f t="shared" si="3"/>
@@ -15478,7 +15475,7 @@
         <v>1022</v>
       </c>
       <c r="N232" s="1" t="s">
-        <v>1415</v>
+        <v>1414</v>
       </c>
       <c r="O232" s="23" t="str">
         <f t="shared" si="3"/>
@@ -15514,7 +15511,7 @@
         <v>1025</v>
       </c>
       <c r="N233" s="1" t="s">
-        <v>1415</v>
+        <v>1414</v>
       </c>
       <c r="O233" s="23" t="str">
         <f t="shared" si="3"/>
@@ -15550,7 +15547,7 @@
         <v>1028</v>
       </c>
       <c r="N234" s="1" t="s">
-        <v>1418</v>
+        <v>1417</v>
       </c>
       <c r="O234" s="23" t="str">
         <f t="shared" si="3"/>
@@ -16270,7 +16267,7 @@
         <v>1049</v>
       </c>
       <c r="N254" s="1" t="s">
-        <v>1421</v>
+        <v>1409</v>
       </c>
       <c r="O254" s="23" t="str">
         <f t="shared" si="3"/>
@@ -16306,7 +16303,7 @@
         <v>1052</v>
       </c>
       <c r="N255" s="1" t="s">
-        <v>1421</v>
+        <v>1409</v>
       </c>
       <c r="O255" s="23" t="str">
         <f t="shared" si="3"/>
@@ -16342,7 +16339,7 @@
         <v>1055</v>
       </c>
       <c r="N256" s="1" t="s">
-        <v>1421</v>
+        <v>1409</v>
       </c>
       <c r="O256" s="23" t="str">
         <f t="shared" si="3"/>
@@ -16378,7 +16375,7 @@
         <v>1058</v>
       </c>
       <c r="N257" s="1" t="s">
-        <v>1427</v>
+        <v>1425</v>
       </c>
       <c r="O257" s="23" t="str">
         <f t="shared" si="3"/>
@@ -16414,7 +16411,7 @@
         <v>1061</v>
       </c>
       <c r="N258" s="1" t="s">
-        <v>1420</v>
+        <v>1419</v>
       </c>
       <c r="O258" s="23" t="str">
         <f t="shared" ref="O258:O320" si="4">"DATA/logos/" &amp; TEXT(E258,"jjj") &amp; ".png"</f>
@@ -16450,7 +16447,7 @@
         <v>1064</v>
       </c>
       <c r="N259" s="1" t="s">
-        <v>1425</v>
+        <v>1423</v>
       </c>
       <c r="O259" s="23" t="str">
         <f t="shared" si="4"/>
@@ -16486,7 +16483,7 @@
         <v>1067</v>
       </c>
       <c r="N260" s="1" t="s">
-        <v>1421</v>
+        <v>1409</v>
       </c>
       <c r="O260" s="23" t="str">
         <f t="shared" si="4"/>
@@ -16522,7 +16519,7 @@
         <v>1070</v>
       </c>
       <c r="N261" s="1" t="s">
-        <v>1424</v>
+        <v>1422</v>
       </c>
       <c r="O261" s="23" t="str">
         <f t="shared" si="4"/>
@@ -16558,7 +16555,7 @@
         <v>1073</v>
       </c>
       <c r="N262" s="1" t="s">
-        <v>1428</v>
+        <v>1426</v>
       </c>
       <c r="O262" s="23" t="str">
         <f t="shared" si="4"/>
@@ -16594,7 +16591,7 @@
         <v>1076</v>
       </c>
       <c r="N263" s="1" t="s">
-        <v>1426</v>
+        <v>1424</v>
       </c>
       <c r="O263" s="23" t="str">
         <f t="shared" si="4"/>
@@ -16630,7 +16627,7 @@
         <v>1079</v>
       </c>
       <c r="N264" s="1" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
       <c r="O264" s="23" t="str">
         <f t="shared" si="4"/>
@@ -16666,7 +16663,7 @@
         <v>1079</v>
       </c>
       <c r="N265" s="1" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
       <c r="O265" s="23" t="str">
         <f t="shared" si="4"/>
@@ -16702,7 +16699,7 @@
         <v>1079</v>
       </c>
       <c r="N266" s="1" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
       <c r="O266" s="23" t="str">
         <f t="shared" si="4"/>
@@ -16738,7 +16735,7 @@
         <v>1084</v>
       </c>
       <c r="N267" s="1" t="s">
-        <v>1429</v>
+        <v>1427</v>
       </c>
       <c r="O267" s="23" t="str">
         <f t="shared" si="4"/>
@@ -16774,7 +16771,7 @@
         <v>1087</v>
       </c>
       <c r="N268" s="1" t="s">
-        <v>1429</v>
+        <v>1427</v>
       </c>
       <c r="O268" s="23" t="str">
         <f t="shared" si="4"/>
@@ -16954,7 +16951,7 @@
         <v>1102</v>
       </c>
       <c r="N273" s="1" t="s">
-        <v>1430</v>
+        <v>1409</v>
       </c>
       <c r="O273" s="23" t="str">
         <f t="shared" si="4"/>
@@ -16990,7 +16987,7 @@
         <v>1105</v>
       </c>
       <c r="N274" s="1" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
       <c r="O274" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17001,7 +16998,7 @@
       <c r="A275" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B275" s="24" t="s">
+      <c r="B275" s="33" t="s">
         <v>119</v>
       </c>
       <c r="C275" s="5" t="s">
@@ -17026,7 +17023,7 @@
         <v>1108</v>
       </c>
       <c r="N275" s="1" t="s">
-        <v>1106</v>
+        <v>1409</v>
       </c>
       <c r="O275" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17098,7 +17095,7 @@
         <v>1004</v>
       </c>
       <c r="N277" s="1" t="s">
-        <v>1420</v>
+        <v>1419</v>
       </c>
       <c r="O277" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17242,7 +17239,7 @@
         <v>1114</v>
       </c>
       <c r="N281" s="1" t="s">
-        <v>1423</v>
+        <v>1421</v>
       </c>
       <c r="O281" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17278,7 +17275,7 @@
         <v>1117</v>
       </c>
       <c r="N282" s="1" t="s">
-        <v>1422</v>
+        <v>1420</v>
       </c>
       <c r="O282" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17314,7 +17311,7 @@
         <v>1120</v>
       </c>
       <c r="N283" s="1" t="s">
-        <v>1414</v>
+        <v>1413</v>
       </c>
       <c r="O283" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17350,7 +17347,7 @@
         <v>1123</v>
       </c>
       <c r="N284" s="1" t="s">
-        <v>1106</v>
+        <v>1409</v>
       </c>
       <c r="O284" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17386,7 +17383,7 @@
         <v>1126</v>
       </c>
       <c r="N285" s="1" t="s">
-        <v>1106</v>
+        <v>1409</v>
       </c>
       <c r="O285" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17422,7 +17419,7 @@
         <v>1129</v>
       </c>
       <c r="N286" s="1" t="s">
-        <v>1421</v>
+        <v>1409</v>
       </c>
       <c r="O286" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17458,7 +17455,7 @@
         <v>-52.289486400000001</v>
       </c>
       <c r="N287" s="1" t="s">
-        <v>1421</v>
+        <v>1409</v>
       </c>
       <c r="O287" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17494,7 +17491,7 @@
         <v>1134</v>
       </c>
       <c r="N288" s="1" t="s">
-        <v>1421</v>
+        <v>1409</v>
       </c>
       <c r="O288" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17530,7 +17527,7 @@
         <v>1137</v>
       </c>
       <c r="N289" s="1" t="s">
-        <v>1420</v>
+        <v>1419</v>
       </c>
       <c r="O289" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17566,7 +17563,7 @@
         <v>1140</v>
       </c>
       <c r="N290" s="1" t="s">
-        <v>1420</v>
+        <v>1419</v>
       </c>
       <c r="O290" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17602,7 +17599,7 @@
         <v>1143</v>
       </c>
       <c r="N291" s="1" t="s">
-        <v>1420</v>
+        <v>1419</v>
       </c>
       <c r="O291" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17638,7 +17635,7 @@
         <v>1146</v>
       </c>
       <c r="N292" s="1" t="s">
-        <v>1417</v>
+        <v>1416</v>
       </c>
       <c r="O292" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17674,7 +17671,7 @@
         <v>1149</v>
       </c>
       <c r="N293" s="1" t="s">
-        <v>1431</v>
+        <v>1409</v>
       </c>
       <c r="O293" s="23" t="str">
         <f t="shared" si="4"/>
@@ -17710,7 +17707,7 @@
         <v>1152</v>
       </c>
       <c r="N294" s="1" t="s">
-        <v>1431</v>
+        <v>1409</v>
       </c>
       <c r="O294" s="23" t="str">
         <f t="shared" si="4"/>
@@ -20500,10 +20497,10 @@
         <v>930</v>
       </c>
       <c r="D372" s="25" t="s">
-        <v>1432</v>
+        <v>1428</v>
       </c>
       <c r="E372" s="25" t="s">
-        <v>1432</v>
+        <v>1428</v>
       </c>
       <c r="F372" s="1"/>
       <c r="G372" s="1"/>
@@ -22149,14 +22146,8 @@
       <c r="M469" s="19"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M380" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Site"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <autoFilter ref="A1:M380" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>